<commit_message>
Waiting Final (Excel sum amount)
</commit_message>
<xml_diff>
--- a/bin/Debug/Template/NGReq_Template.xlsx
+++ b/bin/Debug/Template/NGReq_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\IT-Project\MC-Dept-App\bin\Debug\Template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50269A76-5008-40DD-B2A4-0806C9AB3164}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C57464D1-EF02-40B3-8812-39B39F908D69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6570" yWindow="4650" windowWidth="19185" windowHeight="8640" firstSheet="10" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="10" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="hidden" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1391" uniqueCount="434">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1391" uniqueCount="431">
   <si>
     <t>#</t>
     <phoneticPr fontId="1"/>
@@ -1705,19 +1705,10 @@
     <t>Machine</t>
   </si>
   <si>
-    <t xml:space="preserve"> REF: WH-RE-006  REV:04  Date: 27/01/2025    </t>
-  </si>
-  <si>
     <t>RM Code</t>
   </si>
   <si>
     <t>Note:</t>
-  </si>
-  <si>
-    <t>For Account section will sign this report when each section issue dispose only.</t>
-  </si>
-  <si>
-    <t>For process transfer, return, request please follow normal process, no need acount sign.</t>
   </si>
   <si>
     <t>NG0000000001</t>
@@ -3800,6 +3791,96 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="66" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="56" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="57" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="58" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="59" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="60" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="61" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="59" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="60" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="62" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="63" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="37" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="44" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="64" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="44" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="44" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="19" fillId="0" borderId="45" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -3875,96 +3956,6 @@
     <xf numFmtId="49" fontId="19" fillId="0" borderId="47" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="64" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="44" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="44" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="56" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="57" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="58" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="59" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="60" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="61" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="59" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="60" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="62" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="63" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="37" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="44" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -4003,6 +3994,96 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="64" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="19" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -4079,96 +4160,6 @@
     <xf numFmtId="49" fontId="19" fillId="0" borderId="47" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="64" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -4199,18 +4190,6 @@
     <xf numFmtId="0" fontId="48" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="51" fillId="4" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="49" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="15" fontId="50" fillId="4" borderId="52" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="4" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="50" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -4235,13 +4214,34 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="51" fillId="4" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="49" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="15" fontId="50" fillId="4" borderId="52" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="4" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="48" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
@@ -4259,22 +4259,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="48" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -8020,8 +8011,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="154886" y="1022827"/>
-          <a:ext cx="3438516" cy="1066126"/>
+          <a:off x="154886" y="1024120"/>
+          <a:ext cx="3427741" cy="1071297"/>
           <a:chOff x="154886" y="1022575"/>
           <a:chExt cx="3435737" cy="1065086"/>
         </a:xfrm>
@@ -8764,8 +8755,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="351692" y="2224161"/>
-          <a:ext cx="1901470" cy="509712"/>
+          <a:off x="347382" y="2230195"/>
+          <a:ext cx="1895005" cy="509712"/>
           <a:chOff x="354330" y="2232660"/>
           <a:chExt cx="1901682" cy="509712"/>
         </a:xfrm>
@@ -9101,8 +9092,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="3915613" y="2224161"/>
-          <a:ext cx="2062655" cy="509712"/>
+          <a:off x="3904407" y="2230195"/>
+          <a:ext cx="2059207" cy="509712"/>
           <a:chOff x="354330" y="2232660"/>
           <a:chExt cx="1901682" cy="509712"/>
         </a:xfrm>
@@ -9438,8 +9429,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="7300353" y="2043439"/>
-          <a:ext cx="2193065" cy="681097"/>
+          <a:off x="7286130" y="2048611"/>
+          <a:ext cx="2202547" cy="681959"/>
           <a:chOff x="9976701" y="1996964"/>
           <a:chExt cx="2110196" cy="682603"/>
         </a:xfrm>
@@ -9893,8 +9884,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="52551" y="4032837"/>
-          <a:ext cx="9427731" cy="1140729"/>
+          <a:off x="52551" y="4041457"/>
+          <a:ext cx="9422990" cy="1140298"/>
           <a:chOff x="52551" y="4355224"/>
           <a:chExt cx="7679120" cy="1070743"/>
         </a:xfrm>
@@ -30182,6 +30173,16 @@
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="K9:L9"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="E10:E11"/>
+    <mergeCell ref="G10:H10"/>
+    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="K5:L5"/>
+    <mergeCell ref="I6:J6"/>
     <mergeCell ref="G41:I41"/>
     <mergeCell ref="J36:K36"/>
     <mergeCell ref="C11:D11"/>
@@ -30191,16 +30192,6 @@
     <mergeCell ref="C36:D36"/>
     <mergeCell ref="E36:F36"/>
     <mergeCell ref="G36:I36"/>
-    <mergeCell ref="A3:L3"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="K5:L5"/>
-    <mergeCell ref="I6:J6"/>
-    <mergeCell ref="J9:J10"/>
-    <mergeCell ref="K9:L9"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="E10:E11"/>
-    <mergeCell ref="G10:H10"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.5" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="70" orientation="portrait" r:id="rId1"/>
@@ -30236,10 +30227,10 @@
         <v>142</v>
       </c>
       <c r="I1" s="252" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
       <c r="J1" s="228" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="15.75">
@@ -30248,28 +30239,28 @@
       </c>
     </row>
     <row r="3" spans="1:13" ht="25.5">
-      <c r="A3" s="398" t="s">
+      <c r="A3" s="406" t="s">
         <v>229</v>
       </c>
-      <c r="B3" s="398"/>
-      <c r="C3" s="398"/>
-      <c r="D3" s="398"/>
-      <c r="E3" s="398"/>
-      <c r="F3" s="398"/>
-      <c r="G3" s="398"/>
-      <c r="H3" s="398"/>
-      <c r="I3" s="398"/>
-      <c r="J3" s="398"/>
-      <c r="K3" s="398"/>
-      <c r="L3" s="398"/>
-      <c r="M3" s="398"/>
+      <c r="B3" s="406"/>
+      <c r="C3" s="406"/>
+      <c r="D3" s="406"/>
+      <c r="E3" s="406"/>
+      <c r="F3" s="406"/>
+      <c r="G3" s="406"/>
+      <c r="H3" s="406"/>
+      <c r="I3" s="406"/>
+      <c r="J3" s="406"/>
+      <c r="K3" s="406"/>
+      <c r="L3" s="406"/>
+      <c r="M3" s="406"/>
     </row>
     <row r="4" spans="1:13" ht="20.100000000000001" customHeight="1">
       <c r="I4" s="230" t="s">
         <v>88</v>
       </c>
-      <c r="J4" s="399"/>
-      <c r="K4" s="399"/>
+      <c r="J4" s="407"/>
+      <c r="K4" s="407"/>
       <c r="L4" s="231"/>
       <c r="M4" s="231"/>
     </row>
@@ -30277,19 +30268,19 @@
       <c r="I5" s="230" t="s">
         <v>89</v>
       </c>
-      <c r="J5" s="400"/>
-      <c r="K5" s="400"/>
-      <c r="L5" s="397"/>
-      <c r="M5" s="397"/>
+      <c r="J5" s="408"/>
+      <c r="K5" s="408"/>
+      <c r="L5" s="405"/>
+      <c r="M5" s="405"/>
     </row>
     <row r="6" spans="1:13" ht="20.25" customHeight="1">
       <c r="I6" s="230" t="s">
         <v>90</v>
       </c>
-      <c r="J6" s="400" t="s">
+      <c r="J6" s="408" t="s">
         <v>423</v>
       </c>
-      <c r="K6" s="400"/>
+      <c r="K6" s="408"/>
       <c r="L6" s="232"/>
       <c r="M6" s="232"/>
     </row>
@@ -30297,14 +30288,14 @@
       <c r="I7" s="230" t="s">
         <v>91</v>
       </c>
-      <c r="J7" s="397"/>
-      <c r="K7" s="397"/>
-      <c r="L7" s="397"/>
+      <c r="J7" s="405"/>
+      <c r="K7" s="405"/>
+      <c r="L7" s="405"/>
       <c r="M7" s="232"/>
     </row>
     <row r="8" spans="1:13" ht="20.25" customHeight="1">
       <c r="E8" s="253" t="s">
-        <v>430</v>
+        <v>427</v>
       </c>
       <c r="I8" s="233"/>
       <c r="J8" s="234"/>
@@ -30313,33 +30304,33 @@
       <c r="M8" s="234"/>
     </row>
     <row r="9" spans="1:13" ht="13.5" customHeight="1">
-      <c r="K9" s="407"/>
-      <c r="L9" s="408"/>
-      <c r="M9" s="408"/>
+      <c r="K9" s="403"/>
+      <c r="L9" s="404"/>
+      <c r="M9" s="404"/>
     </row>
     <row r="10" spans="1:13">
       <c r="B10" s="234"/>
-      <c r="C10" s="408"/>
-      <c r="D10" s="408"/>
-      <c r="E10" s="407"/>
+      <c r="C10" s="404"/>
+      <c r="D10" s="404"/>
+      <c r="E10" s="403"/>
       <c r="F10" s="235"/>
       <c r="G10" s="234"/>
-      <c r="H10" s="408"/>
-      <c r="I10" s="408"/>
+      <c r="H10" s="404"/>
+      <c r="I10" s="404"/>
       <c r="J10" s="234"/>
-      <c r="K10" s="407"/>
+      <c r="K10" s="403"/>
       <c r="L10" s="234"/>
       <c r="M10" s="236"/>
     </row>
     <row r="11" spans="1:13" ht="26.25" customHeight="1">
       <c r="B11" s="235"/>
-      <c r="C11" s="407"/>
-      <c r="D11" s="407"/>
-      <c r="E11" s="407"/>
+      <c r="C11" s="403"/>
+      <c r="D11" s="403"/>
+      <c r="E11" s="403"/>
       <c r="F11" s="235"/>
       <c r="G11" s="235"/>
-      <c r="H11" s="407"/>
-      <c r="I11" s="407"/>
+      <c r="H11" s="403"/>
+      <c r="I11" s="403"/>
       <c r="J11" s="234"/>
       <c r="K11" s="234"/>
     </row>
@@ -30355,12 +30346,12 @@
         <v>225</v>
       </c>
       <c r="D13" s="238" t="s">
-        <v>425</v>
-      </c>
-      <c r="E13" s="401" t="s">
+        <v>424</v>
+      </c>
+      <c r="E13" s="397" t="s">
         <v>51</v>
       </c>
-      <c r="F13" s="402"/>
+      <c r="F13" s="398"/>
       <c r="G13" s="238" t="s">
         <v>52</v>
       </c>
@@ -30388,25 +30379,25 @@
       <c r="B14" s="239"/>
       <c r="C14" s="239"/>
       <c r="D14" s="254"/>
-      <c r="E14" s="403"/>
-      <c r="F14" s="404"/>
+      <c r="E14" s="399"/>
+      <c r="F14" s="400"/>
       <c r="G14" s="240"/>
       <c r="H14" s="241"/>
       <c r="I14" s="255"/>
       <c r="J14" s="242"/>
       <c r="K14" s="243"/>
       <c r="L14" s="244" t="s">
-        <v>430</v>
+        <v>427</v>
       </c>
       <c r="M14" s="245"/>
     </row>
     <row r="15" spans="1:13" ht="16.5" customHeight="1">
-      <c r="A15" s="405" t="s">
+      <c r="A15" s="401" t="s">
         <v>392</v>
       </c>
-      <c r="B15" s="406"/>
-      <c r="C15" s="406"/>
-      <c r="D15" s="406"/>
+      <c r="B15" s="402"/>
+      <c r="C15" s="402"/>
+      <c r="D15" s="402"/>
       <c r="E15" s="246"/>
       <c r="F15" s="246"/>
       <c r="G15" s="246"/>
@@ -30423,20 +30414,26 @@
     <row r="16" spans="1:13" ht="13.5" customHeight="1"/>
     <row r="26" spans="4:5">
       <c r="D26" s="250" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="E26" s="251" t="s">
-        <v>432</v>
+        <v>429</v>
       </c>
     </row>
     <row r="27" spans="4:5">
       <c r="D27" s="251"/>
       <c r="E27" s="251" t="s">
-        <v>433</v>
+        <v>430</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="J7:L7"/>
+    <mergeCell ref="A3:M3"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="L5:M5"/>
+    <mergeCell ref="J6:K6"/>
     <mergeCell ref="E13:F13"/>
     <mergeCell ref="E14:F14"/>
     <mergeCell ref="A15:D15"/>
@@ -30447,12 +30444,6 @@
     <mergeCell ref="H10:I10"/>
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="H11:I11"/>
-    <mergeCell ref="J7:L7"/>
-    <mergeCell ref="A3:M3"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="L5:M5"/>
-    <mergeCell ref="J6:K6"/>
   </mergeCells>
   <pageMargins left="0.1" right="0.1" top="0.2" bottom="0.2" header="0.1" footer="0.1"/>
   <pageSetup paperSize="9" scale="71" fitToHeight="0" orientation="portrait" r:id="rId1"/>
@@ -30489,10 +30480,10 @@
         <v>142</v>
       </c>
       <c r="I1" s="252" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
       <c r="J1" s="228" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="15.75">
@@ -30501,28 +30492,28 @@
       </c>
     </row>
     <row r="3" spans="1:13" ht="25.5">
-      <c r="A3" s="398" t="s">
+      <c r="A3" s="406" t="s">
         <v>229</v>
       </c>
-      <c r="B3" s="398"/>
-      <c r="C3" s="398"/>
-      <c r="D3" s="398"/>
-      <c r="E3" s="398"/>
-      <c r="F3" s="398"/>
-      <c r="G3" s="398"/>
-      <c r="H3" s="398"/>
-      <c r="I3" s="398"/>
-      <c r="J3" s="398"/>
-      <c r="K3" s="398"/>
-      <c r="L3" s="398"/>
-      <c r="M3" s="398"/>
+      <c r="B3" s="406"/>
+      <c r="C3" s="406"/>
+      <c r="D3" s="406"/>
+      <c r="E3" s="406"/>
+      <c r="F3" s="406"/>
+      <c r="G3" s="406"/>
+      <c r="H3" s="406"/>
+      <c r="I3" s="406"/>
+      <c r="J3" s="406"/>
+      <c r="K3" s="406"/>
+      <c r="L3" s="406"/>
+      <c r="M3" s="406"/>
     </row>
     <row r="4" spans="1:13" ht="20.100000000000001" customHeight="1">
       <c r="I4" s="230" t="s">
         <v>88</v>
       </c>
-      <c r="J4" s="399"/>
-      <c r="K4" s="399"/>
+      <c r="J4" s="407"/>
+      <c r="K4" s="407"/>
       <c r="L4" s="231"/>
       <c r="M4" s="231"/>
     </row>
@@ -30530,19 +30521,19 @@
       <c r="I5" s="230" t="s">
         <v>89</v>
       </c>
-      <c r="J5" s="400"/>
-      <c r="K5" s="400"/>
-      <c r="L5" s="397"/>
-      <c r="M5" s="397"/>
+      <c r="J5" s="408"/>
+      <c r="K5" s="408"/>
+      <c r="L5" s="405"/>
+      <c r="M5" s="405"/>
     </row>
     <row r="6" spans="1:13" ht="20.25" customHeight="1">
       <c r="I6" s="230" t="s">
         <v>90</v>
       </c>
-      <c r="J6" s="400" t="s">
+      <c r="J6" s="408" t="s">
         <v>423</v>
       </c>
-      <c r="K6" s="400"/>
+      <c r="K6" s="408"/>
       <c r="L6" s="232"/>
       <c r="M6" s="232"/>
     </row>
@@ -30550,14 +30541,14 @@
       <c r="I7" s="230" t="s">
         <v>91</v>
       </c>
-      <c r="J7" s="397"/>
-      <c r="K7" s="397"/>
-      <c r="L7" s="397"/>
+      <c r="J7" s="405"/>
+      <c r="K7" s="405"/>
+      <c r="L7" s="405"/>
       <c r="M7" s="232"/>
     </row>
     <row r="8" spans="1:13" ht="20.25" customHeight="1">
       <c r="E8" s="253" t="s">
-        <v>430</v>
+        <v>427</v>
       </c>
       <c r="I8" s="233"/>
       <c r="J8" s="234"/>
@@ -30566,33 +30557,33 @@
       <c r="M8" s="234"/>
     </row>
     <row r="9" spans="1:13" ht="13.5" customHeight="1">
-      <c r="K9" s="407"/>
-      <c r="L9" s="408"/>
-      <c r="M9" s="408"/>
+      <c r="K9" s="403"/>
+      <c r="L9" s="404"/>
+      <c r="M9" s="404"/>
     </row>
     <row r="10" spans="1:13">
       <c r="B10" s="234"/>
-      <c r="C10" s="408"/>
-      <c r="D10" s="408"/>
-      <c r="E10" s="407"/>
+      <c r="C10" s="404"/>
+      <c r="D10" s="404"/>
+      <c r="E10" s="403"/>
       <c r="F10" s="235"/>
       <c r="G10" s="234"/>
-      <c r="H10" s="408"/>
-      <c r="I10" s="408"/>
+      <c r="H10" s="404"/>
+      <c r="I10" s="404"/>
       <c r="J10" s="234"/>
-      <c r="K10" s="407"/>
+      <c r="K10" s="403"/>
       <c r="L10" s="234"/>
       <c r="M10" s="236"/>
     </row>
     <row r="11" spans="1:13" ht="26.25" customHeight="1">
       <c r="B11" s="235"/>
-      <c r="C11" s="407"/>
-      <c r="D11" s="407"/>
-      <c r="E11" s="407"/>
+      <c r="C11" s="403"/>
+      <c r="D11" s="403"/>
+      <c r="E11" s="403"/>
       <c r="F11" s="235"/>
       <c r="G11" s="235"/>
-      <c r="H11" s="407"/>
-      <c r="I11" s="407"/>
+      <c r="H11" s="403"/>
+      <c r="I11" s="403"/>
       <c r="J11" s="234"/>
       <c r="K11" s="234"/>
     </row>
@@ -30608,12 +30599,12 @@
         <v>225</v>
       </c>
       <c r="D13" s="238" t="s">
-        <v>425</v>
-      </c>
-      <c r="E13" s="401" t="s">
+        <v>424</v>
+      </c>
+      <c r="E13" s="397" t="s">
         <v>51</v>
       </c>
-      <c r="F13" s="402"/>
+      <c r="F13" s="398"/>
       <c r="G13" s="238" t="s">
         <v>52</v>
       </c>
@@ -30641,25 +30632,25 @@
       <c r="B14" s="239"/>
       <c r="C14" s="239"/>
       <c r="D14" s="254"/>
-      <c r="E14" s="403"/>
-      <c r="F14" s="404"/>
+      <c r="E14" s="399"/>
+      <c r="F14" s="400"/>
       <c r="G14" s="240"/>
       <c r="H14" s="241"/>
       <c r="I14" s="255"/>
       <c r="J14" s="242"/>
       <c r="K14" s="243"/>
       <c r="L14" s="244" t="s">
-        <v>430</v>
+        <v>427</v>
       </c>
       <c r="M14" s="245"/>
     </row>
     <row r="15" spans="1:13" ht="16.5" customHeight="1">
-      <c r="A15" s="405" t="s">
+      <c r="A15" s="401" t="s">
         <v>392</v>
       </c>
-      <c r="B15" s="406"/>
-      <c r="C15" s="406"/>
-      <c r="D15" s="406"/>
+      <c r="B15" s="402"/>
+      <c r="C15" s="402"/>
+      <c r="D15" s="402"/>
       <c r="E15" s="246"/>
       <c r="F15" s="246"/>
       <c r="G15" s="246"/>
@@ -30676,26 +30667,20 @@
     <row r="16" spans="1:13" ht="13.5" customHeight="1"/>
     <row r="26" spans="4:5">
       <c r="D26" s="250" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="E26" s="251" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
     </row>
     <row r="27" spans="4:5">
       <c r="D27" s="251"/>
       <c r="E27" s="251" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="J7:L7"/>
-    <mergeCell ref="A3:M3"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="L5:M5"/>
-    <mergeCell ref="J6:K6"/>
     <mergeCell ref="E13:F13"/>
     <mergeCell ref="E14:F14"/>
     <mergeCell ref="A15:D15"/>
@@ -30706,6 +30691,12 @@
     <mergeCell ref="H10:I10"/>
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="H11:I11"/>
+    <mergeCell ref="J7:L7"/>
+    <mergeCell ref="A3:M3"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="L5:M5"/>
+    <mergeCell ref="J6:K6"/>
   </mergeCells>
   <pageMargins left="0.1" right="0.1" top="0.2" bottom="0.2" header="0.1" footer="0.1"/>
   <pageSetup paperSize="9" scale="71" fitToHeight="0" orientation="portrait" r:id="rId1"/>
@@ -30744,18 +30735,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" s="409" t="s">
+      <c r="A1" s="420" t="s">
         <v>48</v>
       </c>
-      <c r="B1" s="409"/>
-      <c r="C1" s="409"/>
-      <c r="D1" s="409"/>
-      <c r="E1" s="409"/>
-      <c r="F1" s="409"/>
-      <c r="G1" s="409"/>
-      <c r="H1" s="409"/>
-      <c r="I1" s="409"/>
-      <c r="J1" s="409"/>
+      <c r="B1" s="420"/>
+      <c r="C1" s="420"/>
+      <c r="D1" s="420"/>
+      <c r="E1" s="420"/>
+      <c r="F1" s="420"/>
+      <c r="G1" s="420"/>
+      <c r="H1" s="420"/>
+      <c r="I1" s="420"/>
+      <c r="J1" s="420"/>
     </row>
     <row r="2" spans="1:10" ht="26.25">
       <c r="A2" s="322" t="s">
@@ -30830,11 +30821,11 @@
       <c r="B10" s="53" t="s">
         <v>50</v>
       </c>
-      <c r="C10" s="410" t="s">
+      <c r="C10" s="421" t="s">
         <v>51</v>
       </c>
-      <c r="D10" s="410"/>
-      <c r="E10" s="410"/>
+      <c r="D10" s="421"/>
+      <c r="E10" s="421"/>
       <c r="F10" s="53" t="s">
         <v>52</v>
       </c>
@@ -30844,24 +30835,24 @@
       <c r="H10" s="53" t="s">
         <v>54</v>
       </c>
-      <c r="I10" s="410" t="s">
+      <c r="I10" s="421" t="s">
         <v>6</v>
       </c>
-      <c r="J10" s="411"/>
+      <c r="J10" s="422"/>
     </row>
     <row r="11" spans="1:10" ht="20.25" customHeight="1" thickTop="1">
       <c r="A11" s="69">
         <v>1</v>
       </c>
       <c r="B11" s="6"/>
-      <c r="C11" s="412"/>
-      <c r="D11" s="413"/>
-      <c r="E11" s="414"/>
+      <c r="C11" s="415"/>
+      <c r="D11" s="416"/>
+      <c r="E11" s="417"/>
       <c r="F11" s="6"/>
       <c r="G11" s="6"/>
       <c r="H11" s="6"/>
-      <c r="I11" s="415"/>
-      <c r="J11" s="416"/>
+      <c r="I11" s="418"/>
+      <c r="J11" s="419"/>
     </row>
     <row r="12" spans="1:10" ht="20.25" customHeight="1">
       <c r="A12" s="70">
@@ -30875,7 +30866,7 @@
       <c r="G12" s="10"/>
       <c r="H12" s="10"/>
       <c r="I12" s="330"/>
-      <c r="J12" s="417"/>
+      <c r="J12" s="414"/>
     </row>
     <row r="13" spans="1:10" ht="20.25" customHeight="1">
       <c r="A13" s="69">
@@ -30889,7 +30880,7 @@
       <c r="G13" s="10"/>
       <c r="H13" s="10"/>
       <c r="I13" s="330"/>
-      <c r="J13" s="417"/>
+      <c r="J13" s="414"/>
     </row>
     <row r="14" spans="1:10" ht="20.25" customHeight="1">
       <c r="A14" s="70">
@@ -30903,7 +30894,7 @@
       <c r="G14" s="10"/>
       <c r="H14" s="10"/>
       <c r="I14" s="330"/>
-      <c r="J14" s="417"/>
+      <c r="J14" s="414"/>
     </row>
     <row r="15" spans="1:10" ht="20.25" customHeight="1">
       <c r="A15" s="69">
@@ -30917,7 +30908,7 @@
       <c r="G15" s="10"/>
       <c r="H15" s="10"/>
       <c r="I15" s="330"/>
-      <c r="J15" s="417"/>
+      <c r="J15" s="414"/>
     </row>
     <row r="16" spans="1:10" ht="20.25" customHeight="1">
       <c r="A16" s="70">
@@ -30931,7 +30922,7 @@
       <c r="G16" s="10"/>
       <c r="H16" s="10"/>
       <c r="I16" s="330"/>
-      <c r="J16" s="417"/>
+      <c r="J16" s="414"/>
     </row>
     <row r="17" spans="1:10" ht="20.25" customHeight="1">
       <c r="A17" s="69">
@@ -30945,7 +30936,7 @@
       <c r="G17" s="10"/>
       <c r="H17" s="10"/>
       <c r="I17" s="330"/>
-      <c r="J17" s="417"/>
+      <c r="J17" s="414"/>
     </row>
     <row r="18" spans="1:10" ht="20.25" customHeight="1">
       <c r="A18" s="70">
@@ -30959,7 +30950,7 @@
       <c r="G18" s="10"/>
       <c r="H18" s="10"/>
       <c r="I18" s="330"/>
-      <c r="J18" s="417"/>
+      <c r="J18" s="414"/>
     </row>
     <row r="19" spans="1:10" ht="20.25" customHeight="1">
       <c r="A19" s="69">
@@ -30973,7 +30964,7 @@
       <c r="G19" s="10"/>
       <c r="H19" s="10"/>
       <c r="I19" s="330"/>
-      <c r="J19" s="417"/>
+      <c r="J19" s="414"/>
     </row>
     <row r="20" spans="1:10" ht="20.25" customHeight="1">
       <c r="A20" s="70">
@@ -30987,7 +30978,7 @@
       <c r="G20" s="10"/>
       <c r="H20" s="10"/>
       <c r="I20" s="330"/>
-      <c r="J20" s="417"/>
+      <c r="J20" s="414"/>
     </row>
     <row r="21" spans="1:10" ht="20.25" customHeight="1">
       <c r="A21" s="69">
@@ -31001,7 +30992,7 @@
       <c r="G21" s="10"/>
       <c r="H21" s="10"/>
       <c r="I21" s="330"/>
-      <c r="J21" s="417"/>
+      <c r="J21" s="414"/>
     </row>
     <row r="22" spans="1:10" ht="20.25" customHeight="1">
       <c r="A22" s="70">
@@ -31015,7 +31006,7 @@
       <c r="G22" s="10"/>
       <c r="H22" s="10"/>
       <c r="I22" s="330"/>
-      <c r="J22" s="417"/>
+      <c r="J22" s="414"/>
     </row>
     <row r="23" spans="1:10" ht="20.25" customHeight="1">
       <c r="A23" s="69">
@@ -31029,7 +31020,7 @@
       <c r="G23" s="10"/>
       <c r="H23" s="10"/>
       <c r="I23" s="330"/>
-      <c r="J23" s="417"/>
+      <c r="J23" s="414"/>
     </row>
     <row r="24" spans="1:10" ht="20.25" customHeight="1">
       <c r="A24" s="70">
@@ -31043,7 +31034,7 @@
       <c r="G24" s="10"/>
       <c r="H24" s="10"/>
       <c r="I24" s="330"/>
-      <c r="J24" s="417"/>
+      <c r="J24" s="414"/>
     </row>
     <row r="25" spans="1:10" ht="20.25" customHeight="1">
       <c r="A25" s="69">
@@ -31057,7 +31048,7 @@
       <c r="G25" s="10"/>
       <c r="H25" s="10"/>
       <c r="I25" s="330"/>
-      <c r="J25" s="417"/>
+      <c r="J25" s="414"/>
     </row>
     <row r="26" spans="1:10" ht="20.25" customHeight="1">
       <c r="A26" s="70">
@@ -31071,7 +31062,7 @@
       <c r="G26" s="10"/>
       <c r="H26" s="10"/>
       <c r="I26" s="330"/>
-      <c r="J26" s="417"/>
+      <c r="J26" s="414"/>
     </row>
     <row r="27" spans="1:10" ht="20.25" customHeight="1">
       <c r="A27" s="69">
@@ -31085,7 +31076,7 @@
       <c r="G27" s="10"/>
       <c r="H27" s="10"/>
       <c r="I27" s="330"/>
-      <c r="J27" s="417"/>
+      <c r="J27" s="414"/>
     </row>
     <row r="28" spans="1:10" ht="20.25" customHeight="1">
       <c r="A28" s="70">
@@ -31099,7 +31090,7 @@
       <c r="G28" s="10"/>
       <c r="H28" s="10"/>
       <c r="I28" s="330"/>
-      <c r="J28" s="417"/>
+      <c r="J28" s="414"/>
     </row>
     <row r="29" spans="1:10" ht="20.25" customHeight="1">
       <c r="A29" s="69">
@@ -31113,7 +31104,7 @@
       <c r="G29" s="10"/>
       <c r="H29" s="10"/>
       <c r="I29" s="330"/>
-      <c r="J29" s="417"/>
+      <c r="J29" s="414"/>
     </row>
     <row r="30" spans="1:10" ht="20.25" customHeight="1">
       <c r="A30" s="70">
@@ -31127,7 +31118,7 @@
       <c r="G30" s="10"/>
       <c r="H30" s="10"/>
       <c r="I30" s="330"/>
-      <c r="J30" s="417"/>
+      <c r="J30" s="414"/>
     </row>
     <row r="31" spans="1:10" ht="20.25" customHeight="1">
       <c r="A31" s="69">
@@ -31141,7 +31132,7 @@
       <c r="G31" s="10"/>
       <c r="H31" s="10"/>
       <c r="I31" s="330"/>
-      <c r="J31" s="417"/>
+      <c r="J31" s="414"/>
     </row>
     <row r="32" spans="1:10" ht="20.25" customHeight="1">
       <c r="A32" s="70">
@@ -31155,7 +31146,7 @@
       <c r="G32" s="10"/>
       <c r="H32" s="10"/>
       <c r="I32" s="330"/>
-      <c r="J32" s="417"/>
+      <c r="J32" s="414"/>
     </row>
     <row r="33" spans="1:10" ht="20.25" customHeight="1">
       <c r="A33" s="69">
@@ -31169,7 +31160,7 @@
       <c r="G33" s="10"/>
       <c r="H33" s="10"/>
       <c r="I33" s="330"/>
-      <c r="J33" s="417"/>
+      <c r="J33" s="414"/>
     </row>
     <row r="34" spans="1:10" ht="20.25" customHeight="1">
       <c r="A34" s="70">
@@ -31183,7 +31174,7 @@
       <c r="G34" s="10"/>
       <c r="H34" s="10"/>
       <c r="I34" s="330"/>
-      <c r="J34" s="417"/>
+      <c r="J34" s="414"/>
     </row>
     <row r="35" spans="1:10" ht="20.25" customHeight="1">
       <c r="A35" s="69">
@@ -31197,7 +31188,7 @@
       <c r="G35" s="10"/>
       <c r="H35" s="10"/>
       <c r="I35" s="330"/>
-      <c r="J35" s="417"/>
+      <c r="J35" s="414"/>
     </row>
     <row r="36" spans="1:10" ht="20.25" customHeight="1">
       <c r="A36" s="69">
@@ -31211,7 +31202,7 @@
       <c r="G36" s="71"/>
       <c r="H36" s="71"/>
       <c r="I36" s="330"/>
-      <c r="J36" s="417"/>
+      <c r="J36" s="414"/>
     </row>
     <row r="37" spans="1:10" ht="20.25" customHeight="1">
       <c r="A37" s="69">
@@ -31225,7 +31216,7 @@
       <c r="G37" s="71"/>
       <c r="H37" s="71"/>
       <c r="I37" s="330"/>
-      <c r="J37" s="417"/>
+      <c r="J37" s="414"/>
     </row>
     <row r="38" spans="1:10" ht="20.25" customHeight="1">
       <c r="A38" s="69">
@@ -31239,7 +31230,7 @@
       <c r="G38" s="71"/>
       <c r="H38" s="71"/>
       <c r="I38" s="330"/>
-      <c r="J38" s="417"/>
+      <c r="J38" s="414"/>
     </row>
     <row r="39" spans="1:10" ht="20.25" customHeight="1">
       <c r="A39" s="69">
@@ -31253,7 +31244,7 @@
       <c r="G39" s="71"/>
       <c r="H39" s="71"/>
       <c r="I39" s="330"/>
-      <c r="J39" s="417"/>
+      <c r="J39" s="414"/>
     </row>
     <row r="40" spans="1:10" ht="20.25" customHeight="1">
       <c r="A40" s="69">
@@ -31267,19 +31258,19 @@
       <c r="G40" s="71"/>
       <c r="H40" s="71"/>
       <c r="I40" s="330"/>
-      <c r="J40" s="417"/>
+      <c r="J40" s="414"/>
     </row>
     <row r="41" spans="1:10" ht="8.25" customHeight="1" thickBot="1">
       <c r="A41" s="54"/>
       <c r="B41" s="55"/>
-      <c r="C41" s="418"/>
-      <c r="D41" s="419"/>
-      <c r="E41" s="420"/>
+      <c r="C41" s="409"/>
+      <c r="D41" s="410"/>
+      <c r="E41" s="411"/>
       <c r="F41" s="55"/>
       <c r="G41" s="55"/>
       <c r="H41" s="55"/>
-      <c r="I41" s="421"/>
-      <c r="J41" s="422"/>
+      <c r="I41" s="412"/>
+      <c r="J41" s="413"/>
     </row>
     <row r="42" spans="1:10" ht="14.25" customHeight="1">
       <c r="C42" s="72"/>
@@ -31389,6 +31380,71 @@
     </row>
   </sheetData>
   <mergeCells count="72">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C10:E10"/>
+    <mergeCell ref="I10:J10"/>
+    <mergeCell ref="C11:E11"/>
+    <mergeCell ref="I11:J11"/>
+    <mergeCell ref="C12:E12"/>
+    <mergeCell ref="I12:J12"/>
+    <mergeCell ref="C13:E13"/>
+    <mergeCell ref="I13:J13"/>
+    <mergeCell ref="C14:E14"/>
+    <mergeCell ref="I14:J14"/>
+    <mergeCell ref="C15:E15"/>
+    <mergeCell ref="I15:J15"/>
+    <mergeCell ref="C16:E16"/>
+    <mergeCell ref="I16:J16"/>
+    <mergeCell ref="C17:E17"/>
+    <mergeCell ref="I17:J17"/>
+    <mergeCell ref="C18:E18"/>
+    <mergeCell ref="I18:J18"/>
+    <mergeCell ref="C19:E19"/>
+    <mergeCell ref="I19:J19"/>
+    <mergeCell ref="C20:E20"/>
+    <mergeCell ref="I20:J20"/>
+    <mergeCell ref="C21:E21"/>
+    <mergeCell ref="I21:J21"/>
+    <mergeCell ref="C22:E22"/>
+    <mergeCell ref="I22:J22"/>
+    <mergeCell ref="C23:E23"/>
+    <mergeCell ref="I23:J23"/>
+    <mergeCell ref="C24:E24"/>
+    <mergeCell ref="I24:J24"/>
+    <mergeCell ref="C25:E25"/>
+    <mergeCell ref="I25:J25"/>
+    <mergeCell ref="C26:E26"/>
+    <mergeCell ref="I26:J26"/>
+    <mergeCell ref="C27:E27"/>
+    <mergeCell ref="I27:J27"/>
+    <mergeCell ref="C28:E28"/>
+    <mergeCell ref="I28:J28"/>
+    <mergeCell ref="C29:E29"/>
+    <mergeCell ref="I29:J29"/>
+    <mergeCell ref="C30:E30"/>
+    <mergeCell ref="I30:J30"/>
+    <mergeCell ref="C31:E31"/>
+    <mergeCell ref="I31:J31"/>
+    <mergeCell ref="C32:E32"/>
+    <mergeCell ref="I32:J32"/>
+    <mergeCell ref="C33:E33"/>
+    <mergeCell ref="I33:J33"/>
+    <mergeCell ref="C34:E34"/>
+    <mergeCell ref="I34:J34"/>
+    <mergeCell ref="C35:E35"/>
+    <mergeCell ref="I35:J35"/>
+    <mergeCell ref="C36:E36"/>
+    <mergeCell ref="I36:J36"/>
+    <mergeCell ref="C37:E37"/>
+    <mergeCell ref="I37:J37"/>
+    <mergeCell ref="C38:E38"/>
+    <mergeCell ref="I38:J38"/>
+    <mergeCell ref="C39:E39"/>
+    <mergeCell ref="I39:J39"/>
+    <mergeCell ref="C40:E40"/>
+    <mergeCell ref="I40:J40"/>
     <mergeCell ref="C41:E41"/>
     <mergeCell ref="I41:J41"/>
     <mergeCell ref="A45:B45"/>
@@ -31396,71 +31452,6 @@
     <mergeCell ref="E45:F45"/>
     <mergeCell ref="G45:H45"/>
     <mergeCell ref="I45:J45"/>
-    <mergeCell ref="C38:E38"/>
-    <mergeCell ref="I38:J38"/>
-    <mergeCell ref="C39:E39"/>
-    <mergeCell ref="I39:J39"/>
-    <mergeCell ref="C40:E40"/>
-    <mergeCell ref="I40:J40"/>
-    <mergeCell ref="C35:E35"/>
-    <mergeCell ref="I35:J35"/>
-    <mergeCell ref="C36:E36"/>
-    <mergeCell ref="I36:J36"/>
-    <mergeCell ref="C37:E37"/>
-    <mergeCell ref="I37:J37"/>
-    <mergeCell ref="C32:E32"/>
-    <mergeCell ref="I32:J32"/>
-    <mergeCell ref="C33:E33"/>
-    <mergeCell ref="I33:J33"/>
-    <mergeCell ref="C34:E34"/>
-    <mergeCell ref="I34:J34"/>
-    <mergeCell ref="C29:E29"/>
-    <mergeCell ref="I29:J29"/>
-    <mergeCell ref="C30:E30"/>
-    <mergeCell ref="I30:J30"/>
-    <mergeCell ref="C31:E31"/>
-    <mergeCell ref="I31:J31"/>
-    <mergeCell ref="C26:E26"/>
-    <mergeCell ref="I26:J26"/>
-    <mergeCell ref="C27:E27"/>
-    <mergeCell ref="I27:J27"/>
-    <mergeCell ref="C28:E28"/>
-    <mergeCell ref="I28:J28"/>
-    <mergeCell ref="C23:E23"/>
-    <mergeCell ref="I23:J23"/>
-    <mergeCell ref="C24:E24"/>
-    <mergeCell ref="I24:J24"/>
-    <mergeCell ref="C25:E25"/>
-    <mergeCell ref="I25:J25"/>
-    <mergeCell ref="C20:E20"/>
-    <mergeCell ref="I20:J20"/>
-    <mergeCell ref="C21:E21"/>
-    <mergeCell ref="I21:J21"/>
-    <mergeCell ref="C22:E22"/>
-    <mergeCell ref="I22:J22"/>
-    <mergeCell ref="C17:E17"/>
-    <mergeCell ref="I17:J17"/>
-    <mergeCell ref="C18:E18"/>
-    <mergeCell ref="I18:J18"/>
-    <mergeCell ref="C19:E19"/>
-    <mergeCell ref="I19:J19"/>
-    <mergeCell ref="C14:E14"/>
-    <mergeCell ref="I14:J14"/>
-    <mergeCell ref="C15:E15"/>
-    <mergeCell ref="I15:J15"/>
-    <mergeCell ref="C16:E16"/>
-    <mergeCell ref="I16:J16"/>
-    <mergeCell ref="C11:E11"/>
-    <mergeCell ref="I11:J11"/>
-    <mergeCell ref="C12:E12"/>
-    <mergeCell ref="I12:J12"/>
-    <mergeCell ref="C13:E13"/>
-    <mergeCell ref="I13:J13"/>
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A2:J2"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C10:E10"/>
-    <mergeCell ref="I10:J10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -34220,152 +34211,152 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="20.25" customHeight="1">
-      <c r="A1" s="301" t="s">
+      <c r="A1" s="264" t="s">
         <v>142</v>
       </c>
-      <c r="B1" s="302"/>
-      <c r="C1" s="302"/>
-      <c r="D1" s="302"/>
-      <c r="E1" s="302"/>
-      <c r="F1" s="302"/>
-      <c r="G1" s="302"/>
-      <c r="H1" s="303"/>
-      <c r="I1" s="304" t="s">
+      <c r="B1" s="265"/>
+      <c r="C1" s="265"/>
+      <c r="D1" s="265"/>
+      <c r="E1" s="265"/>
+      <c r="F1" s="265"/>
+      <c r="G1" s="265"/>
+      <c r="H1" s="266"/>
+      <c r="I1" s="267" t="s">
         <v>143</v>
       </c>
-      <c r="J1" s="305"/>
-      <c r="K1" s="306"/>
-      <c r="L1" s="307" t="s">
+      <c r="J1" s="268"/>
+      <c r="K1" s="269"/>
+      <c r="L1" s="270" t="s">
         <v>144</v>
       </c>
-      <c r="M1" s="308"/>
-      <c r="N1" s="309"/>
+      <c r="M1" s="271"/>
+      <c r="N1" s="272"/>
     </row>
     <row r="2" spans="1:14" ht="30" customHeight="1">
-      <c r="A2" s="310" t="s">
+      <c r="A2" s="273" t="s">
         <v>145</v>
       </c>
-      <c r="B2" s="311"/>
-      <c r="C2" s="311"/>
-      <c r="D2" s="311"/>
-      <c r="E2" s="311"/>
-      <c r="F2" s="311"/>
-      <c r="G2" s="311"/>
-      <c r="H2" s="312"/>
-      <c r="I2" s="313" t="s">
+      <c r="B2" s="274"/>
+      <c r="C2" s="274"/>
+      <c r="D2" s="274"/>
+      <c r="E2" s="274"/>
+      <c r="F2" s="274"/>
+      <c r="G2" s="274"/>
+      <c r="H2" s="275"/>
+      <c r="I2" s="276" t="s">
         <v>146</v>
       </c>
-      <c r="J2" s="314"/>
-      <c r="K2" s="315"/>
-      <c r="L2" s="316" t="s">
+      <c r="J2" s="277"/>
+      <c r="K2" s="278"/>
+      <c r="L2" s="279" t="s">
         <v>147</v>
       </c>
-      <c r="M2" s="317"/>
-      <c r="N2" s="318"/>
+      <c r="M2" s="280"/>
+      <c r="N2" s="281"/>
     </row>
     <row r="3" spans="1:14" ht="30.75" customHeight="1">
-      <c r="A3" s="289" t="s">
+      <c r="A3" s="282" t="s">
         <v>148</v>
       </c>
-      <c r="B3" s="290"/>
-      <c r="C3" s="290"/>
-      <c r="D3" s="290"/>
-      <c r="E3" s="290"/>
-      <c r="F3" s="290"/>
-      <c r="G3" s="290"/>
-      <c r="H3" s="291"/>
-      <c r="I3" s="292" t="s">
+      <c r="B3" s="283"/>
+      <c r="C3" s="283"/>
+      <c r="D3" s="283"/>
+      <c r="E3" s="283"/>
+      <c r="F3" s="283"/>
+      <c r="G3" s="283"/>
+      <c r="H3" s="284"/>
+      <c r="I3" s="285" t="s">
         <v>149</v>
       </c>
-      <c r="J3" s="293"/>
-      <c r="K3" s="292" t="s">
+      <c r="J3" s="286"/>
+      <c r="K3" s="285" t="s">
         <v>150</v>
       </c>
-      <c r="L3" s="293"/>
-      <c r="M3" s="292" t="s">
+      <c r="L3" s="286"/>
+      <c r="M3" s="285" t="s">
         <v>151</v>
       </c>
-      <c r="N3" s="294"/>
+      <c r="N3" s="287"/>
     </row>
     <row r="4" spans="1:14" ht="43.5" customHeight="1">
       <c r="A4" s="85" t="s">
         <v>152</v>
       </c>
-      <c r="B4" s="295" t="s">
+      <c r="B4" s="288" t="s">
         <v>153</v>
       </c>
-      <c r="C4" s="296"/>
-      <c r="D4" s="296"/>
-      <c r="E4" s="296"/>
-      <c r="F4" s="296"/>
-      <c r="G4" s="296"/>
-      <c r="H4" s="297"/>
-      <c r="I4" s="298"/>
-      <c r="J4" s="299"/>
-      <c r="K4" s="298"/>
-      <c r="L4" s="299"/>
-      <c r="M4" s="298"/>
-      <c r="N4" s="300"/>
+      <c r="C4" s="289"/>
+      <c r="D4" s="289"/>
+      <c r="E4" s="289"/>
+      <c r="F4" s="289"/>
+      <c r="G4" s="289"/>
+      <c r="H4" s="290"/>
+      <c r="I4" s="291"/>
+      <c r="J4" s="292"/>
+      <c r="K4" s="291"/>
+      <c r="L4" s="292"/>
+      <c r="M4" s="291"/>
+      <c r="N4" s="293"/>
     </row>
     <row r="5" spans="1:14" s="87" customFormat="1" ht="46.5" customHeight="1">
       <c r="A5" s="86">
         <v>1</v>
       </c>
-      <c r="B5" s="266" t="s">
+      <c r="B5" s="296" t="s">
         <v>154</v>
       </c>
-      <c r="C5" s="267"/>
-      <c r="D5" s="267"/>
-      <c r="E5" s="267"/>
-      <c r="F5" s="267"/>
-      <c r="G5" s="267"/>
-      <c r="H5" s="267"/>
-      <c r="I5" s="267"/>
-      <c r="J5" s="267"/>
-      <c r="K5" s="267"/>
-      <c r="L5" s="267"/>
-      <c r="M5" s="267"/>
-      <c r="N5" s="268"/>
+      <c r="C5" s="297"/>
+      <c r="D5" s="297"/>
+      <c r="E5" s="297"/>
+      <c r="F5" s="297"/>
+      <c r="G5" s="297"/>
+      <c r="H5" s="297"/>
+      <c r="I5" s="297"/>
+      <c r="J5" s="297"/>
+      <c r="K5" s="297"/>
+      <c r="L5" s="297"/>
+      <c r="M5" s="297"/>
+      <c r="N5" s="298"/>
     </row>
     <row r="6" spans="1:14" s="87" customFormat="1" ht="39" customHeight="1">
       <c r="A6" s="88">
         <v>2</v>
       </c>
-      <c r="B6" s="269" t="s">
+      <c r="B6" s="299" t="s">
         <v>155</v>
       </c>
-      <c r="C6" s="270"/>
-      <c r="D6" s="270"/>
-      <c r="E6" s="270"/>
-      <c r="F6" s="270"/>
-      <c r="G6" s="270"/>
-      <c r="H6" s="270"/>
-      <c r="I6" s="270"/>
-      <c r="J6" s="270"/>
-      <c r="K6" s="270"/>
-      <c r="L6" s="270"/>
-      <c r="M6" s="270"/>
-      <c r="N6" s="271"/>
+      <c r="C6" s="300"/>
+      <c r="D6" s="300"/>
+      <c r="E6" s="300"/>
+      <c r="F6" s="300"/>
+      <c r="G6" s="300"/>
+      <c r="H6" s="300"/>
+      <c r="I6" s="300"/>
+      <c r="J6" s="300"/>
+      <c r="K6" s="300"/>
+      <c r="L6" s="300"/>
+      <c r="M6" s="300"/>
+      <c r="N6" s="301"/>
     </row>
     <row r="7" spans="1:14" s="87" customFormat="1" ht="21" customHeight="1">
       <c r="A7" s="89" t="s">
         <v>156</v>
       </c>
-      <c r="B7" s="272" t="s">
+      <c r="B7" s="302" t="s">
         <v>157</v>
       </c>
-      <c r="C7" s="273"/>
-      <c r="D7" s="273"/>
-      <c r="E7" s="273"/>
-      <c r="F7" s="273"/>
-      <c r="G7" s="273"/>
-      <c r="H7" s="273"/>
-      <c r="I7" s="273"/>
-      <c r="J7" s="273"/>
-      <c r="K7" s="273"/>
-      <c r="L7" s="273"/>
-      <c r="M7" s="273"/>
-      <c r="N7" s="274"/>
+      <c r="C7" s="303"/>
+      <c r="D7" s="303"/>
+      <c r="E7" s="303"/>
+      <c r="F7" s="303"/>
+      <c r="G7" s="303"/>
+      <c r="H7" s="303"/>
+      <c r="I7" s="303"/>
+      <c r="J7" s="303"/>
+      <c r="K7" s="303"/>
+      <c r="L7" s="303"/>
+      <c r="M7" s="303"/>
+      <c r="N7" s="304"/>
     </row>
     <row r="8" spans="1:14" s="95" customFormat="1" ht="20.100000000000001" customHeight="1">
       <c r="A8" s="90"/>
@@ -34934,7 +34925,7 @@
       <c r="N42" s="99"/>
     </row>
     <row r="43" spans="1:14" s="123" customFormat="1" ht="18.75" customHeight="1">
-      <c r="A43" s="275" t="s">
+      <c r="A43" s="305" t="s">
         <v>162</v>
       </c>
       <c r="B43" s="116" t="s">
@@ -34942,95 +34933,81 @@
       </c>
       <c r="C43" s="117"/>
       <c r="D43" s="118"/>
-      <c r="E43" s="278"/>
-      <c r="F43" s="279"/>
-      <c r="G43" s="279"/>
-      <c r="H43" s="279"/>
-      <c r="I43" s="279"/>
-      <c r="J43" s="279"/>
+      <c r="E43" s="308"/>
+      <c r="F43" s="309"/>
+      <c r="G43" s="309"/>
+      <c r="H43" s="309"/>
+      <c r="I43" s="309"/>
+      <c r="J43" s="309"/>
       <c r="K43" s="121"/>
       <c r="L43" s="120"/>
       <c r="M43" s="119"/>
       <c r="N43" s="122"/>
     </row>
     <row r="44" spans="1:14" s="123" customFormat="1" ht="18.75" customHeight="1">
-      <c r="A44" s="276"/>
+      <c r="A44" s="306"/>
       <c r="B44" s="124" t="s">
         <v>163</v>
       </c>
       <c r="C44" s="125"/>
       <c r="D44" s="126"/>
-      <c r="E44" s="280"/>
-      <c r="F44" s="281"/>
-      <c r="G44" s="281"/>
-      <c r="H44" s="281"/>
-      <c r="I44" s="281"/>
-      <c r="J44" s="281"/>
+      <c r="E44" s="310"/>
+      <c r="F44" s="311"/>
+      <c r="G44" s="311"/>
+      <c r="H44" s="311"/>
+      <c r="I44" s="311"/>
+      <c r="J44" s="311"/>
       <c r="K44" s="127"/>
       <c r="L44" s="128"/>
       <c r="M44" s="129"/>
       <c r="N44" s="130"/>
     </row>
     <row r="45" spans="1:14" s="123" customFormat="1" ht="18.75" customHeight="1">
-      <c r="A45" s="276"/>
+      <c r="A45" s="306"/>
       <c r="B45" s="131" t="s">
         <v>164</v>
       </c>
       <c r="C45" s="125"/>
       <c r="D45" s="126"/>
-      <c r="E45" s="282"/>
-      <c r="F45" s="283"/>
-      <c r="G45" s="283"/>
-      <c r="H45" s="283"/>
-      <c r="I45" s="283"/>
-      <c r="J45" s="283"/>
+      <c r="E45" s="312"/>
+      <c r="F45" s="313"/>
+      <c r="G45" s="313"/>
+      <c r="H45" s="313"/>
+      <c r="I45" s="313"/>
+      <c r="J45" s="313"/>
       <c r="K45" s="132"/>
       <c r="L45" s="128"/>
       <c r="M45" s="133"/>
       <c r="N45" s="134"/>
     </row>
     <row r="46" spans="1:14" s="123" customFormat="1" ht="25.5" customHeight="1" thickBot="1">
-      <c r="A46" s="277"/>
+      <c r="A46" s="307"/>
       <c r="B46" s="135" t="s">
         <v>165</v>
       </c>
-      <c r="C46" s="284" t="s">
+      <c r="C46" s="314" t="s">
         <v>166</v>
       </c>
-      <c r="D46" s="285"/>
-      <c r="E46" s="286" t="s">
+      <c r="D46" s="315"/>
+      <c r="E46" s="316" t="s">
         <v>167</v>
       </c>
-      <c r="F46" s="287"/>
-      <c r="G46" s="287"/>
-      <c r="H46" s="287"/>
-      <c r="I46" s="287"/>
-      <c r="J46" s="288"/>
-      <c r="K46" s="264" t="s">
+      <c r="F46" s="317"/>
+      <c r="G46" s="317"/>
+      <c r="H46" s="317"/>
+      <c r="I46" s="317"/>
+      <c r="J46" s="318"/>
+      <c r="K46" s="294" t="s">
         <v>168</v>
       </c>
-      <c r="L46" s="288"/>
-      <c r="M46" s="264" t="s">
+      <c r="L46" s="318"/>
+      <c r="M46" s="294" t="s">
         <v>169</v>
       </c>
-      <c r="N46" s="265"/>
+      <c r="N46" s="295"/>
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="I1:K1"/>
-    <mergeCell ref="L1:N1"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="L2:N2"/>
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="I3:J3"/>
-    <mergeCell ref="K3:L3"/>
-    <mergeCell ref="M3:N3"/>
-    <mergeCell ref="B4:H4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="M4:N4"/>
     <mergeCell ref="M46:N46"/>
     <mergeCell ref="B5:N5"/>
     <mergeCell ref="B6:N6"/>
@@ -35042,6 +35019,20 @@
     <mergeCell ref="C46:D46"/>
     <mergeCell ref="E46:J46"/>
     <mergeCell ref="K46:L46"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="I3:J3"/>
+    <mergeCell ref="K3:L3"/>
+    <mergeCell ref="M3:N3"/>
+    <mergeCell ref="B4:H4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="L1:N1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="L2:N2"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
@@ -38287,152 +38278,152 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="20.25" customHeight="1">
-      <c r="A1" s="369" t="s">
+      <c r="A1" s="332" t="s">
         <v>142</v>
       </c>
-      <c r="B1" s="370"/>
-      <c r="C1" s="370"/>
-      <c r="D1" s="370"/>
-      <c r="E1" s="370"/>
-      <c r="F1" s="370"/>
-      <c r="G1" s="370"/>
-      <c r="H1" s="371"/>
-      <c r="I1" s="372" t="s">
+      <c r="B1" s="333"/>
+      <c r="C1" s="333"/>
+      <c r="D1" s="333"/>
+      <c r="E1" s="333"/>
+      <c r="F1" s="333"/>
+      <c r="G1" s="333"/>
+      <c r="H1" s="334"/>
+      <c r="I1" s="335" t="s">
         <v>143</v>
       </c>
-      <c r="J1" s="373"/>
-      <c r="K1" s="374"/>
-      <c r="L1" s="375" t="s">
+      <c r="J1" s="336"/>
+      <c r="K1" s="337"/>
+      <c r="L1" s="338" t="s">
         <v>144</v>
       </c>
-      <c r="M1" s="376"/>
-      <c r="N1" s="377"/>
+      <c r="M1" s="339"/>
+      <c r="N1" s="340"/>
     </row>
     <row r="2" spans="1:14" ht="30" customHeight="1">
-      <c r="A2" s="378" t="s">
+      <c r="A2" s="341" t="s">
         <v>145</v>
       </c>
-      <c r="B2" s="379"/>
-      <c r="C2" s="379"/>
-      <c r="D2" s="379"/>
-      <c r="E2" s="379"/>
-      <c r="F2" s="379"/>
-      <c r="G2" s="379"/>
-      <c r="H2" s="380"/>
-      <c r="I2" s="381" t="s">
+      <c r="B2" s="342"/>
+      <c r="C2" s="342"/>
+      <c r="D2" s="342"/>
+      <c r="E2" s="342"/>
+      <c r="F2" s="342"/>
+      <c r="G2" s="342"/>
+      <c r="H2" s="343"/>
+      <c r="I2" s="344" t="s">
         <v>146</v>
       </c>
-      <c r="J2" s="382"/>
-      <c r="K2" s="383"/>
-      <c r="L2" s="384" t="s">
+      <c r="J2" s="345"/>
+      <c r="K2" s="346"/>
+      <c r="L2" s="347" t="s">
         <v>147</v>
       </c>
-      <c r="M2" s="385"/>
-      <c r="N2" s="386"/>
+      <c r="M2" s="348"/>
+      <c r="N2" s="349"/>
     </row>
     <row r="3" spans="1:14" ht="30.75" customHeight="1">
-      <c r="A3" s="357" t="s">
+      <c r="A3" s="350" t="s">
         <v>148</v>
       </c>
-      <c r="B3" s="358"/>
-      <c r="C3" s="358"/>
-      <c r="D3" s="358"/>
-      <c r="E3" s="358"/>
-      <c r="F3" s="358"/>
-      <c r="G3" s="358"/>
-      <c r="H3" s="359"/>
-      <c r="I3" s="360" t="s">
+      <c r="B3" s="351"/>
+      <c r="C3" s="351"/>
+      <c r="D3" s="351"/>
+      <c r="E3" s="351"/>
+      <c r="F3" s="351"/>
+      <c r="G3" s="351"/>
+      <c r="H3" s="352"/>
+      <c r="I3" s="353" t="s">
         <v>149</v>
       </c>
-      <c r="J3" s="361"/>
-      <c r="K3" s="360" t="s">
+      <c r="J3" s="354"/>
+      <c r="K3" s="353" t="s">
         <v>150</v>
       </c>
-      <c r="L3" s="361"/>
-      <c r="M3" s="360" t="s">
+      <c r="L3" s="354"/>
+      <c r="M3" s="353" t="s">
         <v>151</v>
       </c>
-      <c r="N3" s="362"/>
+      <c r="N3" s="355"/>
     </row>
     <row r="4" spans="1:14" ht="43.5" customHeight="1">
       <c r="A4" s="165" t="s">
         <v>152</v>
       </c>
-      <c r="B4" s="363" t="s">
+      <c r="B4" s="356" t="s">
         <v>153</v>
       </c>
-      <c r="C4" s="364"/>
-      <c r="D4" s="364"/>
-      <c r="E4" s="364"/>
-      <c r="F4" s="364"/>
-      <c r="G4" s="364"/>
-      <c r="H4" s="365"/>
-      <c r="I4" s="366"/>
-      <c r="J4" s="367"/>
-      <c r="K4" s="366"/>
-      <c r="L4" s="367"/>
-      <c r="M4" s="366"/>
-      <c r="N4" s="368"/>
+      <c r="C4" s="357"/>
+      <c r="D4" s="357"/>
+      <c r="E4" s="357"/>
+      <c r="F4" s="357"/>
+      <c r="G4" s="357"/>
+      <c r="H4" s="358"/>
+      <c r="I4" s="359"/>
+      <c r="J4" s="360"/>
+      <c r="K4" s="359"/>
+      <c r="L4" s="360"/>
+      <c r="M4" s="359"/>
+      <c r="N4" s="361"/>
     </row>
     <row r="5" spans="1:14" s="167" customFormat="1" ht="46.5" customHeight="1">
       <c r="A5" s="166">
         <v>1</v>
       </c>
-      <c r="B5" s="334" t="s">
+      <c r="B5" s="364" t="s">
         <v>154</v>
       </c>
-      <c r="C5" s="335"/>
-      <c r="D5" s="335"/>
-      <c r="E5" s="335"/>
-      <c r="F5" s="335"/>
-      <c r="G5" s="335"/>
-      <c r="H5" s="335"/>
-      <c r="I5" s="335"/>
-      <c r="J5" s="335"/>
-      <c r="K5" s="335"/>
-      <c r="L5" s="335"/>
-      <c r="M5" s="335"/>
-      <c r="N5" s="336"/>
+      <c r="C5" s="365"/>
+      <c r="D5" s="365"/>
+      <c r="E5" s="365"/>
+      <c r="F5" s="365"/>
+      <c r="G5" s="365"/>
+      <c r="H5" s="365"/>
+      <c r="I5" s="365"/>
+      <c r="J5" s="365"/>
+      <c r="K5" s="365"/>
+      <c r="L5" s="365"/>
+      <c r="M5" s="365"/>
+      <c r="N5" s="366"/>
     </row>
     <row r="6" spans="1:14" s="167" customFormat="1" ht="39" customHeight="1">
       <c r="A6" s="168">
         <v>2</v>
       </c>
-      <c r="B6" s="337" t="s">
+      <c r="B6" s="367" t="s">
         <v>155</v>
       </c>
-      <c r="C6" s="338"/>
-      <c r="D6" s="338"/>
-      <c r="E6" s="338"/>
-      <c r="F6" s="338"/>
-      <c r="G6" s="338"/>
-      <c r="H6" s="338"/>
-      <c r="I6" s="338"/>
-      <c r="J6" s="338"/>
-      <c r="K6" s="338"/>
-      <c r="L6" s="338"/>
-      <c r="M6" s="338"/>
-      <c r="N6" s="339"/>
+      <c r="C6" s="368"/>
+      <c r="D6" s="368"/>
+      <c r="E6" s="368"/>
+      <c r="F6" s="368"/>
+      <c r="G6" s="368"/>
+      <c r="H6" s="368"/>
+      <c r="I6" s="368"/>
+      <c r="J6" s="368"/>
+      <c r="K6" s="368"/>
+      <c r="L6" s="368"/>
+      <c r="M6" s="368"/>
+      <c r="N6" s="369"/>
     </row>
     <row r="7" spans="1:14" s="167" customFormat="1" ht="21" customHeight="1">
       <c r="A7" s="169" t="s">
         <v>156</v>
       </c>
-      <c r="B7" s="340" t="s">
+      <c r="B7" s="370" t="s">
         <v>157</v>
       </c>
-      <c r="C7" s="341"/>
-      <c r="D7" s="341"/>
-      <c r="E7" s="341"/>
-      <c r="F7" s="341"/>
-      <c r="G7" s="341"/>
-      <c r="H7" s="341"/>
-      <c r="I7" s="341"/>
-      <c r="J7" s="341"/>
-      <c r="K7" s="341"/>
-      <c r="L7" s="341"/>
-      <c r="M7" s="341"/>
-      <c r="N7" s="342"/>
+      <c r="C7" s="371"/>
+      <c r="D7" s="371"/>
+      <c r="E7" s="371"/>
+      <c r="F7" s="371"/>
+      <c r="G7" s="371"/>
+      <c r="H7" s="371"/>
+      <c r="I7" s="371"/>
+      <c r="J7" s="371"/>
+      <c r="K7" s="371"/>
+      <c r="L7" s="371"/>
+      <c r="M7" s="371"/>
+      <c r="N7" s="372"/>
     </row>
     <row r="8" spans="1:14" s="174" customFormat="1" ht="20.100000000000001" customHeight="1">
       <c r="A8" s="170"/>
@@ -39001,7 +38992,7 @@
       <c r="N42" s="178"/>
     </row>
     <row r="43" spans="1:14" s="202" customFormat="1" ht="18.75" customHeight="1">
-      <c r="A43" s="343" t="s">
+      <c r="A43" s="373" t="s">
         <v>162</v>
       </c>
       <c r="B43" s="195" t="s">
@@ -39009,95 +39000,81 @@
       </c>
       <c r="C43" s="196"/>
       <c r="D43" s="197"/>
-      <c r="E43" s="346"/>
-      <c r="F43" s="347"/>
-      <c r="G43" s="347"/>
-      <c r="H43" s="347"/>
-      <c r="I43" s="347"/>
-      <c r="J43" s="347"/>
+      <c r="E43" s="376"/>
+      <c r="F43" s="377"/>
+      <c r="G43" s="377"/>
+      <c r="H43" s="377"/>
+      <c r="I43" s="377"/>
+      <c r="J43" s="377"/>
       <c r="K43" s="200"/>
       <c r="L43" s="199"/>
       <c r="M43" s="198"/>
       <c r="N43" s="201"/>
     </row>
     <row r="44" spans="1:14" s="202" customFormat="1" ht="18.75" customHeight="1">
-      <c r="A44" s="344"/>
+      <c r="A44" s="374"/>
       <c r="B44" s="203" t="s">
         <v>163</v>
       </c>
       <c r="C44" s="204"/>
       <c r="D44" s="205"/>
-      <c r="E44" s="348"/>
-      <c r="F44" s="349"/>
-      <c r="G44" s="349"/>
-      <c r="H44" s="349"/>
-      <c r="I44" s="349"/>
-      <c r="J44" s="349"/>
+      <c r="E44" s="378"/>
+      <c r="F44" s="379"/>
+      <c r="G44" s="379"/>
+      <c r="H44" s="379"/>
+      <c r="I44" s="379"/>
+      <c r="J44" s="379"/>
       <c r="K44" s="206"/>
       <c r="L44" s="207"/>
       <c r="M44" s="208"/>
       <c r="N44" s="209"/>
     </row>
     <row r="45" spans="1:14" s="202" customFormat="1" ht="18.75" customHeight="1">
-      <c r="A45" s="344"/>
+      <c r="A45" s="374"/>
       <c r="B45" s="210" t="s">
         <v>164</v>
       </c>
       <c r="C45" s="204"/>
       <c r="D45" s="205"/>
-      <c r="E45" s="350"/>
-      <c r="F45" s="351"/>
-      <c r="G45" s="351"/>
-      <c r="H45" s="351"/>
-      <c r="I45" s="351"/>
-      <c r="J45" s="351"/>
+      <c r="E45" s="380"/>
+      <c r="F45" s="381"/>
+      <c r="G45" s="381"/>
+      <c r="H45" s="381"/>
+      <c r="I45" s="381"/>
+      <c r="J45" s="381"/>
       <c r="K45" s="211"/>
       <c r="L45" s="207"/>
       <c r="M45" s="212"/>
       <c r="N45" s="213"/>
     </row>
     <row r="46" spans="1:14" s="202" customFormat="1" ht="25.5" customHeight="1" thickBot="1">
-      <c r="A46" s="345"/>
+      <c r="A46" s="375"/>
       <c r="B46" s="214" t="s">
         <v>165</v>
       </c>
-      <c r="C46" s="352" t="s">
+      <c r="C46" s="382" t="s">
         <v>166</v>
       </c>
-      <c r="D46" s="353"/>
-      <c r="E46" s="354" t="s">
+      <c r="D46" s="383"/>
+      <c r="E46" s="384" t="s">
         <v>167</v>
       </c>
-      <c r="F46" s="355"/>
-      <c r="G46" s="355"/>
-      <c r="H46" s="355"/>
-      <c r="I46" s="355"/>
-      <c r="J46" s="356"/>
-      <c r="K46" s="332" t="s">
+      <c r="F46" s="385"/>
+      <c r="G46" s="385"/>
+      <c r="H46" s="385"/>
+      <c r="I46" s="385"/>
+      <c r="J46" s="386"/>
+      <c r="K46" s="362" t="s">
         <v>168</v>
       </c>
-      <c r="L46" s="356"/>
-      <c r="M46" s="332" t="s">
+      <c r="L46" s="386"/>
+      <c r="M46" s="362" t="s">
         <v>169</v>
       </c>
-      <c r="N46" s="333"/>
+      <c r="N46" s="363"/>
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="I1:K1"/>
-    <mergeCell ref="L1:N1"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="L2:N2"/>
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="I3:J3"/>
-    <mergeCell ref="K3:L3"/>
-    <mergeCell ref="M3:N3"/>
-    <mergeCell ref="B4:H4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="M4:N4"/>
     <mergeCell ref="M46:N46"/>
     <mergeCell ref="B5:N5"/>
     <mergeCell ref="B6:N6"/>
@@ -39109,6 +39086,20 @@
     <mergeCell ref="C46:D46"/>
     <mergeCell ref="E46:J46"/>
     <mergeCell ref="K46:L46"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="I3:J3"/>
+    <mergeCell ref="K3:L3"/>
+    <mergeCell ref="M3:N3"/>
+    <mergeCell ref="B4:H4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="L1:N1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="L2:N2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -40728,11 +40719,6 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="A52:B52"/>
-    <mergeCell ref="C52:D52"/>
-    <mergeCell ref="E52:F52"/>
-    <mergeCell ref="G52:I52"/>
-    <mergeCell ref="G57:I57"/>
     <mergeCell ref="A49:B49"/>
     <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:L3"/>
@@ -40746,6 +40732,11 @@
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="G11:H11"/>
     <mergeCell ref="I4:J4"/>
+    <mergeCell ref="A52:B52"/>
+    <mergeCell ref="C52:D52"/>
+    <mergeCell ref="E52:F52"/>
+    <mergeCell ref="G52:I52"/>
+    <mergeCell ref="G57:I57"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="68" orientation="portrait" r:id="rId1"/>
@@ -42693,16 +42684,6 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="J9:J10"/>
-    <mergeCell ref="K9:L9"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="E10:E11"/>
-    <mergeCell ref="G10:H10"/>
-    <mergeCell ref="A3:L3"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="K5:L5"/>
-    <mergeCell ref="I6:J6"/>
     <mergeCell ref="G65:I65"/>
     <mergeCell ref="A58:B58"/>
     <mergeCell ref="C11:D11"/>
@@ -42711,6 +42692,16 @@
     <mergeCell ref="C60:D60"/>
     <mergeCell ref="E60:F60"/>
     <mergeCell ref="G60:I60"/>
+    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="K5:L5"/>
+    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="K9:L9"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="E10:E11"/>
+    <mergeCell ref="G10:H10"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="68" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Change template name and Comlumns value
</commit_message>
<xml_diff>
--- a/bin/Debug/Template/NGReq_Template.xlsx
+++ b/bin/Debug/Template/NGReq_Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\IT-Project\MC-Dept-App\bin\Debug\Template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F1D76D8-888A-4695-99A2-AE1765FD5FD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93935A04-FB12-4DDD-9450-7D782A76C0C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="10" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1391" uniqueCount="431">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1391" uniqueCount="432">
   <si>
     <t>#</t>
     <phoneticPr fontId="1"/>
@@ -1724,6 +1724,9 @@
   </si>
   <si>
     <t>For QC Section: Will sign this report only for WH NG raw materials and NG in field processes.</t>
+  </si>
+  <si>
+    <t>NG Request</t>
   </si>
 </sst>
 </file>
@@ -3791,96 +3794,6 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="66" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="56" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="57" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="58" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="59" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="60" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="61" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="59" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="60" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="62" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="63" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="37" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="44" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="64" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="44" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="44" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="19" fillId="0" borderId="45" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -3956,6 +3869,96 @@
     <xf numFmtId="49" fontId="19" fillId="0" borderId="47" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="64" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="44" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="44" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="56" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="57" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="58" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="59" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="60" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="61" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="59" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="60" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="62" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="63" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="37" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="44" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -3994,96 +3997,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="64" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="19" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -4160,6 +4073,96 @@
     <xf numFmtId="49" fontId="19" fillId="0" borderId="47" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="64" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -4190,6 +4193,18 @@
     <xf numFmtId="0" fontId="48" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="51" fillId="4" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="15" fontId="50" fillId="4" borderId="52" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="4" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="50" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -4214,34 +4229,13 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="51" fillId="4" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="49" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="15" fontId="50" fillId="4" borderId="52" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="4" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="48" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
@@ -4259,13 +4253,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="48" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -30173,16 +30176,6 @@
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="J9:J10"/>
-    <mergeCell ref="K9:L9"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="E10:E11"/>
-    <mergeCell ref="G10:H10"/>
-    <mergeCell ref="A3:L3"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="K5:L5"/>
-    <mergeCell ref="I6:J6"/>
     <mergeCell ref="G41:I41"/>
     <mergeCell ref="J36:K36"/>
     <mergeCell ref="C11:D11"/>
@@ -30192,6 +30185,16 @@
     <mergeCell ref="C36:D36"/>
     <mergeCell ref="E36:F36"/>
     <mergeCell ref="G36:I36"/>
+    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="K5:L5"/>
+    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="K9:L9"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="E10:E11"/>
+    <mergeCell ref="G10:H10"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.5" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="70" orientation="portrait" r:id="rId1"/>
@@ -30239,28 +30242,28 @@
       </c>
     </row>
     <row r="3" spans="1:13" ht="25.5">
-      <c r="A3" s="406" t="s">
+      <c r="A3" s="398" t="s">
         <v>229</v>
       </c>
-      <c r="B3" s="406"/>
-      <c r="C3" s="406"/>
-      <c r="D3" s="406"/>
-      <c r="E3" s="406"/>
-      <c r="F3" s="406"/>
-      <c r="G3" s="406"/>
-      <c r="H3" s="406"/>
-      <c r="I3" s="406"/>
-      <c r="J3" s="406"/>
-      <c r="K3" s="406"/>
-      <c r="L3" s="406"/>
-      <c r="M3" s="406"/>
+      <c r="B3" s="398"/>
+      <c r="C3" s="398"/>
+      <c r="D3" s="398"/>
+      <c r="E3" s="398"/>
+      <c r="F3" s="398"/>
+      <c r="G3" s="398"/>
+      <c r="H3" s="398"/>
+      <c r="I3" s="398"/>
+      <c r="J3" s="398"/>
+      <c r="K3" s="398"/>
+      <c r="L3" s="398"/>
+      <c r="M3" s="398"/>
     </row>
     <row r="4" spans="1:13" ht="20.100000000000001" customHeight="1">
       <c r="I4" s="230" t="s">
         <v>88</v>
       </c>
-      <c r="J4" s="407"/>
-      <c r="K4" s="407"/>
+      <c r="J4" s="399"/>
+      <c r="K4" s="399"/>
       <c r="L4" s="231"/>
       <c r="M4" s="231"/>
     </row>
@@ -30268,19 +30271,19 @@
       <c r="I5" s="230" t="s">
         <v>89</v>
       </c>
-      <c r="J5" s="408"/>
-      <c r="K5" s="408"/>
-      <c r="L5" s="405"/>
-      <c r="M5" s="405"/>
+      <c r="J5" s="400"/>
+      <c r="K5" s="400"/>
+      <c r="L5" s="397"/>
+      <c r="M5" s="397"/>
     </row>
     <row r="6" spans="1:13" ht="20.25" customHeight="1">
       <c r="I6" s="230" t="s">
         <v>90</v>
       </c>
-      <c r="J6" s="408" t="s">
+      <c r="J6" s="400" t="s">
         <v>423</v>
       </c>
-      <c r="K6" s="408"/>
+      <c r="K6" s="400"/>
       <c r="L6" s="232"/>
       <c r="M6" s="232"/>
     </row>
@@ -30288,9 +30291,9 @@
       <c r="I7" s="230" t="s">
         <v>91</v>
       </c>
-      <c r="J7" s="405"/>
-      <c r="K7" s="405"/>
-      <c r="L7" s="405"/>
+      <c r="J7" s="397"/>
+      <c r="K7" s="397"/>
+      <c r="L7" s="397"/>
       <c r="M7" s="232"/>
     </row>
     <row r="8" spans="1:13" ht="20.25" customHeight="1">
@@ -30304,33 +30307,33 @@
       <c r="M8" s="234"/>
     </row>
     <row r="9" spans="1:13" ht="13.5" customHeight="1">
-      <c r="K9" s="403"/>
-      <c r="L9" s="404"/>
-      <c r="M9" s="404"/>
+      <c r="K9" s="407"/>
+      <c r="L9" s="408"/>
+      <c r="M9" s="408"/>
     </row>
     <row r="10" spans="1:13">
       <c r="B10" s="234"/>
-      <c r="C10" s="404"/>
-      <c r="D10" s="404"/>
-      <c r="E10" s="403"/>
+      <c r="C10" s="408"/>
+      <c r="D10" s="408"/>
+      <c r="E10" s="407"/>
       <c r="F10" s="235"/>
       <c r="G10" s="234"/>
-      <c r="H10" s="404"/>
-      <c r="I10" s="404"/>
+      <c r="H10" s="408"/>
+      <c r="I10" s="408"/>
       <c r="J10" s="234"/>
-      <c r="K10" s="403"/>
+      <c r="K10" s="407"/>
       <c r="L10" s="234"/>
       <c r="M10" s="236"/>
     </row>
     <row r="11" spans="1:13" ht="26.25" customHeight="1">
       <c r="B11" s="235"/>
-      <c r="C11" s="403"/>
-      <c r="D11" s="403"/>
-      <c r="E11" s="403"/>
+      <c r="C11" s="407"/>
+      <c r="D11" s="407"/>
+      <c r="E11" s="407"/>
       <c r="F11" s="235"/>
       <c r="G11" s="235"/>
-      <c r="H11" s="403"/>
-      <c r="I11" s="403"/>
+      <c r="H11" s="407"/>
+      <c r="I11" s="407"/>
       <c r="J11" s="234"/>
       <c r="K11" s="234"/>
     </row>
@@ -30348,10 +30351,10 @@
       <c r="D13" s="238" t="s">
         <v>424</v>
       </c>
-      <c r="E13" s="397" t="s">
+      <c r="E13" s="401" t="s">
         <v>51</v>
       </c>
-      <c r="F13" s="398"/>
+      <c r="F13" s="402"/>
       <c r="G13" s="238" t="s">
         <v>52</v>
       </c>
@@ -30379,8 +30382,8 @@
       <c r="B14" s="239"/>
       <c r="C14" s="239"/>
       <c r="D14" s="254"/>
-      <c r="E14" s="399"/>
-      <c r="F14" s="400"/>
+      <c r="E14" s="403"/>
+      <c r="F14" s="404"/>
       <c r="G14" s="240"/>
       <c r="H14" s="241"/>
       <c r="I14" s="255"/>
@@ -30392,12 +30395,12 @@
       <c r="M14" s="245"/>
     </row>
     <row r="15" spans="1:13" ht="16.5" customHeight="1">
-      <c r="A15" s="401" t="s">
+      <c r="A15" s="405" t="s">
         <v>392</v>
       </c>
-      <c r="B15" s="402"/>
-      <c r="C15" s="402"/>
-      <c r="D15" s="402"/>
+      <c r="B15" s="406"/>
+      <c r="C15" s="406"/>
+      <c r="D15" s="406"/>
       <c r="E15" s="246"/>
       <c r="F15" s="246"/>
       <c r="G15" s="246"/>
@@ -30428,12 +30431,6 @@
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="J7:L7"/>
-    <mergeCell ref="A3:M3"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="L5:M5"/>
-    <mergeCell ref="J6:K6"/>
     <mergeCell ref="E13:F13"/>
     <mergeCell ref="E14:F14"/>
     <mergeCell ref="A15:D15"/>
@@ -30444,6 +30441,12 @@
     <mergeCell ref="H10:I10"/>
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="H11:I11"/>
+    <mergeCell ref="J7:L7"/>
+    <mergeCell ref="A3:M3"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="L5:M5"/>
+    <mergeCell ref="J6:K6"/>
   </mergeCells>
   <pageMargins left="0.1" right="0.1" top="0.2" bottom="0.2" header="0.1" footer="0.1"/>
   <pageSetup paperSize="9" scale="71" fitToHeight="0" orientation="portrait" r:id="rId1"/>
@@ -30492,28 +30495,28 @@
       </c>
     </row>
     <row r="3" spans="1:13" ht="25.5">
-      <c r="A3" s="406" t="s">
+      <c r="A3" s="398" t="s">
         <v>229</v>
       </c>
-      <c r="B3" s="406"/>
-      <c r="C3" s="406"/>
-      <c r="D3" s="406"/>
-      <c r="E3" s="406"/>
-      <c r="F3" s="406"/>
-      <c r="G3" s="406"/>
-      <c r="H3" s="406"/>
-      <c r="I3" s="406"/>
-      <c r="J3" s="406"/>
-      <c r="K3" s="406"/>
-      <c r="L3" s="406"/>
-      <c r="M3" s="406"/>
+      <c r="B3" s="398"/>
+      <c r="C3" s="398"/>
+      <c r="D3" s="398"/>
+      <c r="E3" s="398"/>
+      <c r="F3" s="398"/>
+      <c r="G3" s="398"/>
+      <c r="H3" s="398"/>
+      <c r="I3" s="398"/>
+      <c r="J3" s="398"/>
+      <c r="K3" s="398"/>
+      <c r="L3" s="398"/>
+      <c r="M3" s="398"/>
     </row>
     <row r="4" spans="1:13" ht="20.100000000000001" customHeight="1">
       <c r="I4" s="230" t="s">
         <v>88</v>
       </c>
-      <c r="J4" s="407"/>
-      <c r="K4" s="407"/>
+      <c r="J4" s="399"/>
+      <c r="K4" s="399"/>
       <c r="L4" s="231"/>
       <c r="M4" s="231"/>
     </row>
@@ -30521,19 +30524,19 @@
       <c r="I5" s="230" t="s">
         <v>89</v>
       </c>
-      <c r="J5" s="408"/>
-      <c r="K5" s="408"/>
-      <c r="L5" s="405"/>
-      <c r="M5" s="405"/>
+      <c r="J5" s="400"/>
+      <c r="K5" s="400"/>
+      <c r="L5" s="397"/>
+      <c r="M5" s="397"/>
     </row>
     <row r="6" spans="1:13" ht="20.25" customHeight="1">
       <c r="I6" s="230" t="s">
         <v>90</v>
       </c>
-      <c r="J6" s="408" t="s">
+      <c r="J6" s="400" t="s">
         <v>423</v>
       </c>
-      <c r="K6" s="408"/>
+      <c r="K6" s="400"/>
       <c r="L6" s="232"/>
       <c r="M6" s="232"/>
     </row>
@@ -30541,9 +30544,9 @@
       <c r="I7" s="230" t="s">
         <v>91</v>
       </c>
-      <c r="J7" s="405"/>
-      <c r="K7" s="405"/>
-      <c r="L7" s="405"/>
+      <c r="J7" s="397"/>
+      <c r="K7" s="397"/>
+      <c r="L7" s="397"/>
       <c r="M7" s="232"/>
     </row>
     <row r="8" spans="1:13" ht="20.25" customHeight="1">
@@ -30557,33 +30560,33 @@
       <c r="M8" s="234"/>
     </row>
     <row r="9" spans="1:13" ht="13.5" customHeight="1">
-      <c r="K9" s="403"/>
-      <c r="L9" s="404"/>
-      <c r="M9" s="404"/>
+      <c r="K9" s="407"/>
+      <c r="L9" s="408"/>
+      <c r="M9" s="408"/>
     </row>
     <row r="10" spans="1:13">
       <c r="B10" s="234"/>
-      <c r="C10" s="404"/>
-      <c r="D10" s="404"/>
-      <c r="E10" s="403"/>
+      <c r="C10" s="408"/>
+      <c r="D10" s="408"/>
+      <c r="E10" s="407"/>
       <c r="F10" s="235"/>
       <c r="G10" s="234"/>
-      <c r="H10" s="404"/>
-      <c r="I10" s="404"/>
+      <c r="H10" s="408"/>
+      <c r="I10" s="408"/>
       <c r="J10" s="234"/>
-      <c r="K10" s="403"/>
+      <c r="K10" s="407"/>
       <c r="L10" s="234"/>
       <c r="M10" s="236"/>
     </row>
     <row r="11" spans="1:13" ht="26.25" customHeight="1">
       <c r="B11" s="235"/>
-      <c r="C11" s="403"/>
-      <c r="D11" s="403"/>
-      <c r="E11" s="403"/>
+      <c r="C11" s="407"/>
+      <c r="D11" s="407"/>
+      <c r="E11" s="407"/>
       <c r="F11" s="235"/>
       <c r="G11" s="235"/>
-      <c r="H11" s="403"/>
-      <c r="I11" s="403"/>
+      <c r="H11" s="407"/>
+      <c r="I11" s="407"/>
       <c r="J11" s="234"/>
       <c r="K11" s="234"/>
     </row>
@@ -30601,10 +30604,10 @@
       <c r="D13" s="238" t="s">
         <v>424</v>
       </c>
-      <c r="E13" s="397" t="s">
+      <c r="E13" s="401" t="s">
         <v>51</v>
       </c>
-      <c r="F13" s="398"/>
+      <c r="F13" s="402"/>
       <c r="G13" s="238" t="s">
         <v>52</v>
       </c>
@@ -30632,25 +30635,25 @@
       <c r="B14" s="239"/>
       <c r="C14" s="239"/>
       <c r="D14" s="254"/>
-      <c r="E14" s="399"/>
-      <c r="F14" s="400"/>
+      <c r="E14" s="403"/>
+      <c r="F14" s="404"/>
       <c r="G14" s="240"/>
       <c r="H14" s="241"/>
       <c r="I14" s="255"/>
       <c r="J14" s="242"/>
       <c r="K14" s="243"/>
       <c r="L14" s="244" t="s">
-        <v>427</v>
+        <v>431</v>
       </c>
       <c r="M14" s="245"/>
     </row>
     <row r="15" spans="1:13" ht="16.5" customHeight="1">
-      <c r="A15" s="401" t="s">
+      <c r="A15" s="405" t="s">
         <v>392</v>
       </c>
-      <c r="B15" s="402"/>
-      <c r="C15" s="402"/>
-      <c r="D15" s="402"/>
+      <c r="B15" s="406"/>
+      <c r="C15" s="406"/>
+      <c r="D15" s="406"/>
       <c r="E15" s="246"/>
       <c r="F15" s="246"/>
       <c r="G15" s="246"/>
@@ -30681,6 +30684,12 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="J7:L7"/>
+    <mergeCell ref="A3:M3"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="L5:M5"/>
+    <mergeCell ref="J6:K6"/>
     <mergeCell ref="E13:F13"/>
     <mergeCell ref="E14:F14"/>
     <mergeCell ref="A15:D15"/>
@@ -30691,12 +30700,6 @@
     <mergeCell ref="H10:I10"/>
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="H11:I11"/>
-    <mergeCell ref="J7:L7"/>
-    <mergeCell ref="A3:M3"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="L5:M5"/>
-    <mergeCell ref="J6:K6"/>
   </mergeCells>
   <pageMargins left="0.1" right="0.1" top="0.2" bottom="0.2" header="0.1" footer="0.1"/>
   <pageSetup paperSize="9" scale="71" fitToHeight="0" orientation="portrait" r:id="rId1"/>
@@ -30735,18 +30738,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" s="420" t="s">
+      <c r="A1" s="409" t="s">
         <v>48</v>
       </c>
-      <c r="B1" s="420"/>
-      <c r="C1" s="420"/>
-      <c r="D1" s="420"/>
-      <c r="E1" s="420"/>
-      <c r="F1" s="420"/>
-      <c r="G1" s="420"/>
-      <c r="H1" s="420"/>
-      <c r="I1" s="420"/>
-      <c r="J1" s="420"/>
+      <c r="B1" s="409"/>
+      <c r="C1" s="409"/>
+      <c r="D1" s="409"/>
+      <c r="E1" s="409"/>
+      <c r="F1" s="409"/>
+      <c r="G1" s="409"/>
+      <c r="H1" s="409"/>
+      <c r="I1" s="409"/>
+      <c r="J1" s="409"/>
     </row>
     <row r="2" spans="1:10" ht="26.25">
       <c r="A2" s="322" t="s">
@@ -30821,11 +30824,11 @@
       <c r="B10" s="53" t="s">
         <v>50</v>
       </c>
-      <c r="C10" s="421" t="s">
+      <c r="C10" s="410" t="s">
         <v>51</v>
       </c>
-      <c r="D10" s="421"/>
-      <c r="E10" s="421"/>
+      <c r="D10" s="410"/>
+      <c r="E10" s="410"/>
       <c r="F10" s="53" t="s">
         <v>52</v>
       </c>
@@ -30835,24 +30838,24 @@
       <c r="H10" s="53" t="s">
         <v>54</v>
       </c>
-      <c r="I10" s="421" t="s">
+      <c r="I10" s="410" t="s">
         <v>6</v>
       </c>
-      <c r="J10" s="422"/>
+      <c r="J10" s="411"/>
     </row>
     <row r="11" spans="1:10" ht="20.25" customHeight="1" thickTop="1">
       <c r="A11" s="69">
         <v>1</v>
       </c>
       <c r="B11" s="6"/>
-      <c r="C11" s="415"/>
-      <c r="D11" s="416"/>
-      <c r="E11" s="417"/>
+      <c r="C11" s="412"/>
+      <c r="D11" s="413"/>
+      <c r="E11" s="414"/>
       <c r="F11" s="6"/>
       <c r="G11" s="6"/>
       <c r="H11" s="6"/>
-      <c r="I11" s="418"/>
-      <c r="J11" s="419"/>
+      <c r="I11" s="415"/>
+      <c r="J11" s="416"/>
     </row>
     <row r="12" spans="1:10" ht="20.25" customHeight="1">
       <c r="A12" s="70">
@@ -30866,7 +30869,7 @@
       <c r="G12" s="10"/>
       <c r="H12" s="10"/>
       <c r="I12" s="330"/>
-      <c r="J12" s="414"/>
+      <c r="J12" s="417"/>
     </row>
     <row r="13" spans="1:10" ht="20.25" customHeight="1">
       <c r="A13" s="69">
@@ -30880,7 +30883,7 @@
       <c r="G13" s="10"/>
       <c r="H13" s="10"/>
       <c r="I13" s="330"/>
-      <c r="J13" s="414"/>
+      <c r="J13" s="417"/>
     </row>
     <row r="14" spans="1:10" ht="20.25" customHeight="1">
       <c r="A14" s="70">
@@ -30894,7 +30897,7 @@
       <c r="G14" s="10"/>
       <c r="H14" s="10"/>
       <c r="I14" s="330"/>
-      <c r="J14" s="414"/>
+      <c r="J14" s="417"/>
     </row>
     <row r="15" spans="1:10" ht="20.25" customHeight="1">
       <c r="A15" s="69">
@@ -30908,7 +30911,7 @@
       <c r="G15" s="10"/>
       <c r="H15" s="10"/>
       <c r="I15" s="330"/>
-      <c r="J15" s="414"/>
+      <c r="J15" s="417"/>
     </row>
     <row r="16" spans="1:10" ht="20.25" customHeight="1">
       <c r="A16" s="70">
@@ -30922,7 +30925,7 @@
       <c r="G16" s="10"/>
       <c r="H16" s="10"/>
       <c r="I16" s="330"/>
-      <c r="J16" s="414"/>
+      <c r="J16" s="417"/>
     </row>
     <row r="17" spans="1:10" ht="20.25" customHeight="1">
       <c r="A17" s="69">
@@ -30936,7 +30939,7 @@
       <c r="G17" s="10"/>
       <c r="H17" s="10"/>
       <c r="I17" s="330"/>
-      <c r="J17" s="414"/>
+      <c r="J17" s="417"/>
     </row>
     <row r="18" spans="1:10" ht="20.25" customHeight="1">
       <c r="A18" s="70">
@@ -30950,7 +30953,7 @@
       <c r="G18" s="10"/>
       <c r="H18" s="10"/>
       <c r="I18" s="330"/>
-      <c r="J18" s="414"/>
+      <c r="J18" s="417"/>
     </row>
     <row r="19" spans="1:10" ht="20.25" customHeight="1">
       <c r="A19" s="69">
@@ -30964,7 +30967,7 @@
       <c r="G19" s="10"/>
       <c r="H19" s="10"/>
       <c r="I19" s="330"/>
-      <c r="J19" s="414"/>
+      <c r="J19" s="417"/>
     </row>
     <row r="20" spans="1:10" ht="20.25" customHeight="1">
       <c r="A20" s="70">
@@ -30978,7 +30981,7 @@
       <c r="G20" s="10"/>
       <c r="H20" s="10"/>
       <c r="I20" s="330"/>
-      <c r="J20" s="414"/>
+      <c r="J20" s="417"/>
     </row>
     <row r="21" spans="1:10" ht="20.25" customHeight="1">
       <c r="A21" s="69">
@@ -30992,7 +30995,7 @@
       <c r="G21" s="10"/>
       <c r="H21" s="10"/>
       <c r="I21" s="330"/>
-      <c r="J21" s="414"/>
+      <c r="J21" s="417"/>
     </row>
     <row r="22" spans="1:10" ht="20.25" customHeight="1">
       <c r="A22" s="70">
@@ -31006,7 +31009,7 @@
       <c r="G22" s="10"/>
       <c r="H22" s="10"/>
       <c r="I22" s="330"/>
-      <c r="J22" s="414"/>
+      <c r="J22" s="417"/>
     </row>
     <row r="23" spans="1:10" ht="20.25" customHeight="1">
       <c r="A23" s="69">
@@ -31020,7 +31023,7 @@
       <c r="G23" s="10"/>
       <c r="H23" s="10"/>
       <c r="I23" s="330"/>
-      <c r="J23" s="414"/>
+      <c r="J23" s="417"/>
     </row>
     <row r="24" spans="1:10" ht="20.25" customHeight="1">
       <c r="A24" s="70">
@@ -31034,7 +31037,7 @@
       <c r="G24" s="10"/>
       <c r="H24" s="10"/>
       <c r="I24" s="330"/>
-      <c r="J24" s="414"/>
+      <c r="J24" s="417"/>
     </row>
     <row r="25" spans="1:10" ht="20.25" customHeight="1">
       <c r="A25" s="69">
@@ -31048,7 +31051,7 @@
       <c r="G25" s="10"/>
       <c r="H25" s="10"/>
       <c r="I25" s="330"/>
-      <c r="J25" s="414"/>
+      <c r="J25" s="417"/>
     </row>
     <row r="26" spans="1:10" ht="20.25" customHeight="1">
       <c r="A26" s="70">
@@ -31062,7 +31065,7 @@
       <c r="G26" s="10"/>
       <c r="H26" s="10"/>
       <c r="I26" s="330"/>
-      <c r="J26" s="414"/>
+      <c r="J26" s="417"/>
     </row>
     <row r="27" spans="1:10" ht="20.25" customHeight="1">
       <c r="A27" s="69">
@@ -31076,7 +31079,7 @@
       <c r="G27" s="10"/>
       <c r="H27" s="10"/>
       <c r="I27" s="330"/>
-      <c r="J27" s="414"/>
+      <c r="J27" s="417"/>
     </row>
     <row r="28" spans="1:10" ht="20.25" customHeight="1">
       <c r="A28" s="70">
@@ -31090,7 +31093,7 @@
       <c r="G28" s="10"/>
       <c r="H28" s="10"/>
       <c r="I28" s="330"/>
-      <c r="J28" s="414"/>
+      <c r="J28" s="417"/>
     </row>
     <row r="29" spans="1:10" ht="20.25" customHeight="1">
       <c r="A29" s="69">
@@ -31104,7 +31107,7 @@
       <c r="G29" s="10"/>
       <c r="H29" s="10"/>
       <c r="I29" s="330"/>
-      <c r="J29" s="414"/>
+      <c r="J29" s="417"/>
     </row>
     <row r="30" spans="1:10" ht="20.25" customHeight="1">
       <c r="A30" s="70">
@@ -31118,7 +31121,7 @@
       <c r="G30" s="10"/>
       <c r="H30" s="10"/>
       <c r="I30" s="330"/>
-      <c r="J30" s="414"/>
+      <c r="J30" s="417"/>
     </row>
     <row r="31" spans="1:10" ht="20.25" customHeight="1">
       <c r="A31" s="69">
@@ -31132,7 +31135,7 @@
       <c r="G31" s="10"/>
       <c r="H31" s="10"/>
       <c r="I31" s="330"/>
-      <c r="J31" s="414"/>
+      <c r="J31" s="417"/>
     </row>
     <row r="32" spans="1:10" ht="20.25" customHeight="1">
       <c r="A32" s="70">
@@ -31146,7 +31149,7 @@
       <c r="G32" s="10"/>
       <c r="H32" s="10"/>
       <c r="I32" s="330"/>
-      <c r="J32" s="414"/>
+      <c r="J32" s="417"/>
     </row>
     <row r="33" spans="1:10" ht="20.25" customHeight="1">
       <c r="A33" s="69">
@@ -31160,7 +31163,7 @@
       <c r="G33" s="10"/>
       <c r="H33" s="10"/>
       <c r="I33" s="330"/>
-      <c r="J33" s="414"/>
+      <c r="J33" s="417"/>
     </row>
     <row r="34" spans="1:10" ht="20.25" customHeight="1">
       <c r="A34" s="70">
@@ -31174,7 +31177,7 @@
       <c r="G34" s="10"/>
       <c r="H34" s="10"/>
       <c r="I34" s="330"/>
-      <c r="J34" s="414"/>
+      <c r="J34" s="417"/>
     </row>
     <row r="35" spans="1:10" ht="20.25" customHeight="1">
       <c r="A35" s="69">
@@ -31188,7 +31191,7 @@
       <c r="G35" s="10"/>
       <c r="H35" s="10"/>
       <c r="I35" s="330"/>
-      <c r="J35" s="414"/>
+      <c r="J35" s="417"/>
     </row>
     <row r="36" spans="1:10" ht="20.25" customHeight="1">
       <c r="A36" s="69">
@@ -31202,7 +31205,7 @@
       <c r="G36" s="71"/>
       <c r="H36" s="71"/>
       <c r="I36" s="330"/>
-      <c r="J36" s="414"/>
+      <c r="J36" s="417"/>
     </row>
     <row r="37" spans="1:10" ht="20.25" customHeight="1">
       <c r="A37" s="69">
@@ -31216,7 +31219,7 @@
       <c r="G37" s="71"/>
       <c r="H37" s="71"/>
       <c r="I37" s="330"/>
-      <c r="J37" s="414"/>
+      <c r="J37" s="417"/>
     </row>
     <row r="38" spans="1:10" ht="20.25" customHeight="1">
       <c r="A38" s="69">
@@ -31230,7 +31233,7 @@
       <c r="G38" s="71"/>
       <c r="H38" s="71"/>
       <c r="I38" s="330"/>
-      <c r="J38" s="414"/>
+      <c r="J38" s="417"/>
     </row>
     <row r="39" spans="1:10" ht="20.25" customHeight="1">
       <c r="A39" s="69">
@@ -31244,7 +31247,7 @@
       <c r="G39" s="71"/>
       <c r="H39" s="71"/>
       <c r="I39" s="330"/>
-      <c r="J39" s="414"/>
+      <c r="J39" s="417"/>
     </row>
     <row r="40" spans="1:10" ht="20.25" customHeight="1">
       <c r="A40" s="69">
@@ -31258,19 +31261,19 @@
       <c r="G40" s="71"/>
       <c r="H40" s="71"/>
       <c r="I40" s="330"/>
-      <c r="J40" s="414"/>
+      <c r="J40" s="417"/>
     </row>
     <row r="41" spans="1:10" ht="8.25" customHeight="1" thickBot="1">
       <c r="A41" s="54"/>
       <c r="B41" s="55"/>
-      <c r="C41" s="409"/>
-      <c r="D41" s="410"/>
-      <c r="E41" s="411"/>
+      <c r="C41" s="418"/>
+      <c r="D41" s="419"/>
+      <c r="E41" s="420"/>
       <c r="F41" s="55"/>
       <c r="G41" s="55"/>
       <c r="H41" s="55"/>
-      <c r="I41" s="412"/>
-      <c r="J41" s="413"/>
+      <c r="I41" s="421"/>
+      <c r="J41" s="422"/>
     </row>
     <row r="42" spans="1:10" ht="14.25" customHeight="1">
       <c r="C42" s="72"/>
@@ -31380,71 +31383,6 @@
     </row>
   </sheetData>
   <mergeCells count="72">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A2:J2"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C10:E10"/>
-    <mergeCell ref="I10:J10"/>
-    <mergeCell ref="C11:E11"/>
-    <mergeCell ref="I11:J11"/>
-    <mergeCell ref="C12:E12"/>
-    <mergeCell ref="I12:J12"/>
-    <mergeCell ref="C13:E13"/>
-    <mergeCell ref="I13:J13"/>
-    <mergeCell ref="C14:E14"/>
-    <mergeCell ref="I14:J14"/>
-    <mergeCell ref="C15:E15"/>
-    <mergeCell ref="I15:J15"/>
-    <mergeCell ref="C16:E16"/>
-    <mergeCell ref="I16:J16"/>
-    <mergeCell ref="C17:E17"/>
-    <mergeCell ref="I17:J17"/>
-    <mergeCell ref="C18:E18"/>
-    <mergeCell ref="I18:J18"/>
-    <mergeCell ref="C19:E19"/>
-    <mergeCell ref="I19:J19"/>
-    <mergeCell ref="C20:E20"/>
-    <mergeCell ref="I20:J20"/>
-    <mergeCell ref="C21:E21"/>
-    <mergeCell ref="I21:J21"/>
-    <mergeCell ref="C22:E22"/>
-    <mergeCell ref="I22:J22"/>
-    <mergeCell ref="C23:E23"/>
-    <mergeCell ref="I23:J23"/>
-    <mergeCell ref="C24:E24"/>
-    <mergeCell ref="I24:J24"/>
-    <mergeCell ref="C25:E25"/>
-    <mergeCell ref="I25:J25"/>
-    <mergeCell ref="C26:E26"/>
-    <mergeCell ref="I26:J26"/>
-    <mergeCell ref="C27:E27"/>
-    <mergeCell ref="I27:J27"/>
-    <mergeCell ref="C28:E28"/>
-    <mergeCell ref="I28:J28"/>
-    <mergeCell ref="C29:E29"/>
-    <mergeCell ref="I29:J29"/>
-    <mergeCell ref="C30:E30"/>
-    <mergeCell ref="I30:J30"/>
-    <mergeCell ref="C31:E31"/>
-    <mergeCell ref="I31:J31"/>
-    <mergeCell ref="C32:E32"/>
-    <mergeCell ref="I32:J32"/>
-    <mergeCell ref="C33:E33"/>
-    <mergeCell ref="I33:J33"/>
-    <mergeCell ref="C34:E34"/>
-    <mergeCell ref="I34:J34"/>
-    <mergeCell ref="C35:E35"/>
-    <mergeCell ref="I35:J35"/>
-    <mergeCell ref="C36:E36"/>
-    <mergeCell ref="I36:J36"/>
-    <mergeCell ref="C37:E37"/>
-    <mergeCell ref="I37:J37"/>
-    <mergeCell ref="C38:E38"/>
-    <mergeCell ref="I38:J38"/>
-    <mergeCell ref="C39:E39"/>
-    <mergeCell ref="I39:J39"/>
-    <mergeCell ref="C40:E40"/>
-    <mergeCell ref="I40:J40"/>
     <mergeCell ref="C41:E41"/>
     <mergeCell ref="I41:J41"/>
     <mergeCell ref="A45:B45"/>
@@ -31452,6 +31390,71 @@
     <mergeCell ref="E45:F45"/>
     <mergeCell ref="G45:H45"/>
     <mergeCell ref="I45:J45"/>
+    <mergeCell ref="C38:E38"/>
+    <mergeCell ref="I38:J38"/>
+    <mergeCell ref="C39:E39"/>
+    <mergeCell ref="I39:J39"/>
+    <mergeCell ref="C40:E40"/>
+    <mergeCell ref="I40:J40"/>
+    <mergeCell ref="C35:E35"/>
+    <mergeCell ref="I35:J35"/>
+    <mergeCell ref="C36:E36"/>
+    <mergeCell ref="I36:J36"/>
+    <mergeCell ref="C37:E37"/>
+    <mergeCell ref="I37:J37"/>
+    <mergeCell ref="C32:E32"/>
+    <mergeCell ref="I32:J32"/>
+    <mergeCell ref="C33:E33"/>
+    <mergeCell ref="I33:J33"/>
+    <mergeCell ref="C34:E34"/>
+    <mergeCell ref="I34:J34"/>
+    <mergeCell ref="C29:E29"/>
+    <mergeCell ref="I29:J29"/>
+    <mergeCell ref="C30:E30"/>
+    <mergeCell ref="I30:J30"/>
+    <mergeCell ref="C31:E31"/>
+    <mergeCell ref="I31:J31"/>
+    <mergeCell ref="C26:E26"/>
+    <mergeCell ref="I26:J26"/>
+    <mergeCell ref="C27:E27"/>
+    <mergeCell ref="I27:J27"/>
+    <mergeCell ref="C28:E28"/>
+    <mergeCell ref="I28:J28"/>
+    <mergeCell ref="C23:E23"/>
+    <mergeCell ref="I23:J23"/>
+    <mergeCell ref="C24:E24"/>
+    <mergeCell ref="I24:J24"/>
+    <mergeCell ref="C25:E25"/>
+    <mergeCell ref="I25:J25"/>
+    <mergeCell ref="C20:E20"/>
+    <mergeCell ref="I20:J20"/>
+    <mergeCell ref="C21:E21"/>
+    <mergeCell ref="I21:J21"/>
+    <mergeCell ref="C22:E22"/>
+    <mergeCell ref="I22:J22"/>
+    <mergeCell ref="C17:E17"/>
+    <mergeCell ref="I17:J17"/>
+    <mergeCell ref="C18:E18"/>
+    <mergeCell ref="I18:J18"/>
+    <mergeCell ref="C19:E19"/>
+    <mergeCell ref="I19:J19"/>
+    <mergeCell ref="C14:E14"/>
+    <mergeCell ref="I14:J14"/>
+    <mergeCell ref="C15:E15"/>
+    <mergeCell ref="I15:J15"/>
+    <mergeCell ref="C16:E16"/>
+    <mergeCell ref="I16:J16"/>
+    <mergeCell ref="C11:E11"/>
+    <mergeCell ref="I11:J11"/>
+    <mergeCell ref="C12:E12"/>
+    <mergeCell ref="I12:J12"/>
+    <mergeCell ref="C13:E13"/>
+    <mergeCell ref="I13:J13"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C10:E10"/>
+    <mergeCell ref="I10:J10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -34211,152 +34214,152 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="20.25" customHeight="1">
-      <c r="A1" s="264" t="s">
+      <c r="A1" s="301" t="s">
         <v>142</v>
       </c>
-      <c r="B1" s="265"/>
-      <c r="C1" s="265"/>
-      <c r="D1" s="265"/>
-      <c r="E1" s="265"/>
-      <c r="F1" s="265"/>
-      <c r="G1" s="265"/>
-      <c r="H1" s="266"/>
-      <c r="I1" s="267" t="s">
+      <c r="B1" s="302"/>
+      <c r="C1" s="302"/>
+      <c r="D1" s="302"/>
+      <c r="E1" s="302"/>
+      <c r="F1" s="302"/>
+      <c r="G1" s="302"/>
+      <c r="H1" s="303"/>
+      <c r="I1" s="304" t="s">
         <v>143</v>
       </c>
-      <c r="J1" s="268"/>
-      <c r="K1" s="269"/>
-      <c r="L1" s="270" t="s">
+      <c r="J1" s="305"/>
+      <c r="K1" s="306"/>
+      <c r="L1" s="307" t="s">
         <v>144</v>
       </c>
-      <c r="M1" s="271"/>
-      <c r="N1" s="272"/>
+      <c r="M1" s="308"/>
+      <c r="N1" s="309"/>
     </row>
     <row r="2" spans="1:14" ht="30" customHeight="1">
-      <c r="A2" s="273" t="s">
+      <c r="A2" s="310" t="s">
         <v>145</v>
       </c>
-      <c r="B2" s="274"/>
-      <c r="C2" s="274"/>
-      <c r="D2" s="274"/>
-      <c r="E2" s="274"/>
-      <c r="F2" s="274"/>
-      <c r="G2" s="274"/>
-      <c r="H2" s="275"/>
-      <c r="I2" s="276" t="s">
+      <c r="B2" s="311"/>
+      <c r="C2" s="311"/>
+      <c r="D2" s="311"/>
+      <c r="E2" s="311"/>
+      <c r="F2" s="311"/>
+      <c r="G2" s="311"/>
+      <c r="H2" s="312"/>
+      <c r="I2" s="313" t="s">
         <v>146</v>
       </c>
-      <c r="J2" s="277"/>
-      <c r="K2" s="278"/>
-      <c r="L2" s="279" t="s">
+      <c r="J2" s="314"/>
+      <c r="K2" s="315"/>
+      <c r="L2" s="316" t="s">
         <v>147</v>
       </c>
-      <c r="M2" s="280"/>
-      <c r="N2" s="281"/>
+      <c r="M2" s="317"/>
+      <c r="N2" s="318"/>
     </row>
     <row r="3" spans="1:14" ht="30.75" customHeight="1">
-      <c r="A3" s="282" t="s">
+      <c r="A3" s="289" t="s">
         <v>148</v>
       </c>
-      <c r="B3" s="283"/>
-      <c r="C3" s="283"/>
-      <c r="D3" s="283"/>
-      <c r="E3" s="283"/>
-      <c r="F3" s="283"/>
-      <c r="G3" s="283"/>
-      <c r="H3" s="284"/>
-      <c r="I3" s="285" t="s">
+      <c r="B3" s="290"/>
+      <c r="C3" s="290"/>
+      <c r="D3" s="290"/>
+      <c r="E3" s="290"/>
+      <c r="F3" s="290"/>
+      <c r="G3" s="290"/>
+      <c r="H3" s="291"/>
+      <c r="I3" s="292" t="s">
         <v>149</v>
       </c>
-      <c r="J3" s="286"/>
-      <c r="K3" s="285" t="s">
+      <c r="J3" s="293"/>
+      <c r="K3" s="292" t="s">
         <v>150</v>
       </c>
-      <c r="L3" s="286"/>
-      <c r="M3" s="285" t="s">
+      <c r="L3" s="293"/>
+      <c r="M3" s="292" t="s">
         <v>151</v>
       </c>
-      <c r="N3" s="287"/>
+      <c r="N3" s="294"/>
     </row>
     <row r="4" spans="1:14" ht="43.5" customHeight="1">
       <c r="A4" s="85" t="s">
         <v>152</v>
       </c>
-      <c r="B4" s="288" t="s">
+      <c r="B4" s="295" t="s">
         <v>153</v>
       </c>
-      <c r="C4" s="289"/>
-      <c r="D4" s="289"/>
-      <c r="E4" s="289"/>
-      <c r="F4" s="289"/>
-      <c r="G4" s="289"/>
-      <c r="H4" s="290"/>
-      <c r="I4" s="291"/>
-      <c r="J4" s="292"/>
-      <c r="K4" s="291"/>
-      <c r="L4" s="292"/>
-      <c r="M4" s="291"/>
-      <c r="N4" s="293"/>
+      <c r="C4" s="296"/>
+      <c r="D4" s="296"/>
+      <c r="E4" s="296"/>
+      <c r="F4" s="296"/>
+      <c r="G4" s="296"/>
+      <c r="H4" s="297"/>
+      <c r="I4" s="298"/>
+      <c r="J4" s="299"/>
+      <c r="K4" s="298"/>
+      <c r="L4" s="299"/>
+      <c r="M4" s="298"/>
+      <c r="N4" s="300"/>
     </row>
     <row r="5" spans="1:14" s="87" customFormat="1" ht="46.5" customHeight="1">
       <c r="A5" s="86">
         <v>1</v>
       </c>
-      <c r="B5" s="296" t="s">
+      <c r="B5" s="266" t="s">
         <v>154</v>
       </c>
-      <c r="C5" s="297"/>
-      <c r="D5" s="297"/>
-      <c r="E5" s="297"/>
-      <c r="F5" s="297"/>
-      <c r="G5" s="297"/>
-      <c r="H5" s="297"/>
-      <c r="I5" s="297"/>
-      <c r="J5" s="297"/>
-      <c r="K5" s="297"/>
-      <c r="L5" s="297"/>
-      <c r="M5" s="297"/>
-      <c r="N5" s="298"/>
+      <c r="C5" s="267"/>
+      <c r="D5" s="267"/>
+      <c r="E5" s="267"/>
+      <c r="F5" s="267"/>
+      <c r="G5" s="267"/>
+      <c r="H5" s="267"/>
+      <c r="I5" s="267"/>
+      <c r="J5" s="267"/>
+      <c r="K5" s="267"/>
+      <c r="L5" s="267"/>
+      <c r="M5" s="267"/>
+      <c r="N5" s="268"/>
     </row>
     <row r="6" spans="1:14" s="87" customFormat="1" ht="39" customHeight="1">
       <c r="A6" s="88">
         <v>2</v>
       </c>
-      <c r="B6" s="299" t="s">
+      <c r="B6" s="269" t="s">
         <v>155</v>
       </c>
-      <c r="C6" s="300"/>
-      <c r="D6" s="300"/>
-      <c r="E6" s="300"/>
-      <c r="F6" s="300"/>
-      <c r="G6" s="300"/>
-      <c r="H6" s="300"/>
-      <c r="I6" s="300"/>
-      <c r="J6" s="300"/>
-      <c r="K6" s="300"/>
-      <c r="L6" s="300"/>
-      <c r="M6" s="300"/>
-      <c r="N6" s="301"/>
+      <c r="C6" s="270"/>
+      <c r="D6" s="270"/>
+      <c r="E6" s="270"/>
+      <c r="F6" s="270"/>
+      <c r="G6" s="270"/>
+      <c r="H6" s="270"/>
+      <c r="I6" s="270"/>
+      <c r="J6" s="270"/>
+      <c r="K6" s="270"/>
+      <c r="L6" s="270"/>
+      <c r="M6" s="270"/>
+      <c r="N6" s="271"/>
     </row>
     <row r="7" spans="1:14" s="87" customFormat="1" ht="21" customHeight="1">
       <c r="A7" s="89" t="s">
         <v>156</v>
       </c>
-      <c r="B7" s="302" t="s">
+      <c r="B7" s="272" t="s">
         <v>157</v>
       </c>
-      <c r="C7" s="303"/>
-      <c r="D7" s="303"/>
-      <c r="E7" s="303"/>
-      <c r="F7" s="303"/>
-      <c r="G7" s="303"/>
-      <c r="H7" s="303"/>
-      <c r="I7" s="303"/>
-      <c r="J7" s="303"/>
-      <c r="K7" s="303"/>
-      <c r="L7" s="303"/>
-      <c r="M7" s="303"/>
-      <c r="N7" s="304"/>
+      <c r="C7" s="273"/>
+      <c r="D7" s="273"/>
+      <c r="E7" s="273"/>
+      <c r="F7" s="273"/>
+      <c r="G7" s="273"/>
+      <c r="H7" s="273"/>
+      <c r="I7" s="273"/>
+      <c r="J7" s="273"/>
+      <c r="K7" s="273"/>
+      <c r="L7" s="273"/>
+      <c r="M7" s="273"/>
+      <c r="N7" s="274"/>
     </row>
     <row r="8" spans="1:14" s="95" customFormat="1" ht="20.100000000000001" customHeight="1">
       <c r="A8" s="90"/>
@@ -34925,7 +34928,7 @@
       <c r="N42" s="99"/>
     </row>
     <row r="43" spans="1:14" s="123" customFormat="1" ht="18.75" customHeight="1">
-      <c r="A43" s="305" t="s">
+      <c r="A43" s="275" t="s">
         <v>162</v>
       </c>
       <c r="B43" s="116" t="s">
@@ -34933,81 +34936,95 @@
       </c>
       <c r="C43" s="117"/>
       <c r="D43" s="118"/>
-      <c r="E43" s="308"/>
-      <c r="F43" s="309"/>
-      <c r="G43" s="309"/>
-      <c r="H43" s="309"/>
-      <c r="I43" s="309"/>
-      <c r="J43" s="309"/>
+      <c r="E43" s="278"/>
+      <c r="F43" s="279"/>
+      <c r="G43" s="279"/>
+      <c r="H43" s="279"/>
+      <c r="I43" s="279"/>
+      <c r="J43" s="279"/>
       <c r="K43" s="121"/>
       <c r="L43" s="120"/>
       <c r="M43" s="119"/>
       <c r="N43" s="122"/>
     </row>
     <row r="44" spans="1:14" s="123" customFormat="1" ht="18.75" customHeight="1">
-      <c r="A44" s="306"/>
+      <c r="A44" s="276"/>
       <c r="B44" s="124" t="s">
         <v>163</v>
       </c>
       <c r="C44" s="125"/>
       <c r="D44" s="126"/>
-      <c r="E44" s="310"/>
-      <c r="F44" s="311"/>
-      <c r="G44" s="311"/>
-      <c r="H44" s="311"/>
-      <c r="I44" s="311"/>
-      <c r="J44" s="311"/>
+      <c r="E44" s="280"/>
+      <c r="F44" s="281"/>
+      <c r="G44" s="281"/>
+      <c r="H44" s="281"/>
+      <c r="I44" s="281"/>
+      <c r="J44" s="281"/>
       <c r="K44" s="127"/>
       <c r="L44" s="128"/>
       <c r="M44" s="129"/>
       <c r="N44" s="130"/>
     </row>
     <row r="45" spans="1:14" s="123" customFormat="1" ht="18.75" customHeight="1">
-      <c r="A45" s="306"/>
+      <c r="A45" s="276"/>
       <c r="B45" s="131" t="s">
         <v>164</v>
       </c>
       <c r="C45" s="125"/>
       <c r="D45" s="126"/>
-      <c r="E45" s="312"/>
-      <c r="F45" s="313"/>
-      <c r="G45" s="313"/>
-      <c r="H45" s="313"/>
-      <c r="I45" s="313"/>
-      <c r="J45" s="313"/>
+      <c r="E45" s="282"/>
+      <c r="F45" s="283"/>
+      <c r="G45" s="283"/>
+      <c r="H45" s="283"/>
+      <c r="I45" s="283"/>
+      <c r="J45" s="283"/>
       <c r="K45" s="132"/>
       <c r="L45" s="128"/>
       <c r="M45" s="133"/>
       <c r="N45" s="134"/>
     </row>
     <row r="46" spans="1:14" s="123" customFormat="1" ht="25.5" customHeight="1" thickBot="1">
-      <c r="A46" s="307"/>
+      <c r="A46" s="277"/>
       <c r="B46" s="135" t="s">
         <v>165</v>
       </c>
-      <c r="C46" s="314" t="s">
+      <c r="C46" s="284" t="s">
         <v>166</v>
       </c>
-      <c r="D46" s="315"/>
-      <c r="E46" s="316" t="s">
+      <c r="D46" s="285"/>
+      <c r="E46" s="286" t="s">
         <v>167</v>
       </c>
-      <c r="F46" s="317"/>
-      <c r="G46" s="317"/>
-      <c r="H46" s="317"/>
-      <c r="I46" s="317"/>
-      <c r="J46" s="318"/>
-      <c r="K46" s="294" t="s">
+      <c r="F46" s="287"/>
+      <c r="G46" s="287"/>
+      <c r="H46" s="287"/>
+      <c r="I46" s="287"/>
+      <c r="J46" s="288"/>
+      <c r="K46" s="264" t="s">
         <v>168</v>
       </c>
-      <c r="L46" s="318"/>
-      <c r="M46" s="294" t="s">
+      <c r="L46" s="288"/>
+      <c r="M46" s="264" t="s">
         <v>169</v>
       </c>
-      <c r="N46" s="295"/>
+      <c r="N46" s="265"/>
     </row>
   </sheetData>
   <mergeCells count="25">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="L1:N1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="L2:N2"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="I3:J3"/>
+    <mergeCell ref="K3:L3"/>
+    <mergeCell ref="M3:N3"/>
+    <mergeCell ref="B4:H4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="M4:N4"/>
     <mergeCell ref="M46:N46"/>
     <mergeCell ref="B5:N5"/>
     <mergeCell ref="B6:N6"/>
@@ -35019,20 +35036,6 @@
     <mergeCell ref="C46:D46"/>
     <mergeCell ref="E46:J46"/>
     <mergeCell ref="K46:L46"/>
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="I3:J3"/>
-    <mergeCell ref="K3:L3"/>
-    <mergeCell ref="M3:N3"/>
-    <mergeCell ref="B4:H4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="M4:N4"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="I1:K1"/>
-    <mergeCell ref="L1:N1"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="L2:N2"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
@@ -38278,152 +38281,152 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="20.25" customHeight="1">
-      <c r="A1" s="332" t="s">
+      <c r="A1" s="369" t="s">
         <v>142</v>
       </c>
-      <c r="B1" s="333"/>
-      <c r="C1" s="333"/>
-      <c r="D1" s="333"/>
-      <c r="E1" s="333"/>
-      <c r="F1" s="333"/>
-      <c r="G1" s="333"/>
-      <c r="H1" s="334"/>
-      <c r="I1" s="335" t="s">
+      <c r="B1" s="370"/>
+      <c r="C1" s="370"/>
+      <c r="D1" s="370"/>
+      <c r="E1" s="370"/>
+      <c r="F1" s="370"/>
+      <c r="G1" s="370"/>
+      <c r="H1" s="371"/>
+      <c r="I1" s="372" t="s">
         <v>143</v>
       </c>
-      <c r="J1" s="336"/>
-      <c r="K1" s="337"/>
-      <c r="L1" s="338" t="s">
+      <c r="J1" s="373"/>
+      <c r="K1" s="374"/>
+      <c r="L1" s="375" t="s">
         <v>144</v>
       </c>
-      <c r="M1" s="339"/>
-      <c r="N1" s="340"/>
+      <c r="M1" s="376"/>
+      <c r="N1" s="377"/>
     </row>
     <row r="2" spans="1:14" ht="30" customHeight="1">
-      <c r="A2" s="341" t="s">
+      <c r="A2" s="378" t="s">
         <v>145</v>
       </c>
-      <c r="B2" s="342"/>
-      <c r="C2" s="342"/>
-      <c r="D2" s="342"/>
-      <c r="E2" s="342"/>
-      <c r="F2" s="342"/>
-      <c r="G2" s="342"/>
-      <c r="H2" s="343"/>
-      <c r="I2" s="344" t="s">
+      <c r="B2" s="379"/>
+      <c r="C2" s="379"/>
+      <c r="D2" s="379"/>
+      <c r="E2" s="379"/>
+      <c r="F2" s="379"/>
+      <c r="G2" s="379"/>
+      <c r="H2" s="380"/>
+      <c r="I2" s="381" t="s">
         <v>146</v>
       </c>
-      <c r="J2" s="345"/>
-      <c r="K2" s="346"/>
-      <c r="L2" s="347" t="s">
+      <c r="J2" s="382"/>
+      <c r="K2" s="383"/>
+      <c r="L2" s="384" t="s">
         <v>147</v>
       </c>
-      <c r="M2" s="348"/>
-      <c r="N2" s="349"/>
+      <c r="M2" s="385"/>
+      <c r="N2" s="386"/>
     </row>
     <row r="3" spans="1:14" ht="30.75" customHeight="1">
-      <c r="A3" s="350" t="s">
+      <c r="A3" s="357" t="s">
         <v>148</v>
       </c>
-      <c r="B3" s="351"/>
-      <c r="C3" s="351"/>
-      <c r="D3" s="351"/>
-      <c r="E3" s="351"/>
-      <c r="F3" s="351"/>
-      <c r="G3" s="351"/>
-      <c r="H3" s="352"/>
-      <c r="I3" s="353" t="s">
+      <c r="B3" s="358"/>
+      <c r="C3" s="358"/>
+      <c r="D3" s="358"/>
+      <c r="E3" s="358"/>
+      <c r="F3" s="358"/>
+      <c r="G3" s="358"/>
+      <c r="H3" s="359"/>
+      <c r="I3" s="360" t="s">
         <v>149</v>
       </c>
-      <c r="J3" s="354"/>
-      <c r="K3" s="353" t="s">
+      <c r="J3" s="361"/>
+      <c r="K3" s="360" t="s">
         <v>150</v>
       </c>
-      <c r="L3" s="354"/>
-      <c r="M3" s="353" t="s">
+      <c r="L3" s="361"/>
+      <c r="M3" s="360" t="s">
         <v>151</v>
       </c>
-      <c r="N3" s="355"/>
+      <c r="N3" s="362"/>
     </row>
     <row r="4" spans="1:14" ht="43.5" customHeight="1">
       <c r="A4" s="165" t="s">
         <v>152</v>
       </c>
-      <c r="B4" s="356" t="s">
+      <c r="B4" s="363" t="s">
         <v>153</v>
       </c>
-      <c r="C4" s="357"/>
-      <c r="D4" s="357"/>
-      <c r="E4" s="357"/>
-      <c r="F4" s="357"/>
-      <c r="G4" s="357"/>
-      <c r="H4" s="358"/>
-      <c r="I4" s="359"/>
-      <c r="J4" s="360"/>
-      <c r="K4" s="359"/>
-      <c r="L4" s="360"/>
-      <c r="M4" s="359"/>
-      <c r="N4" s="361"/>
+      <c r="C4" s="364"/>
+      <c r="D4" s="364"/>
+      <c r="E4" s="364"/>
+      <c r="F4" s="364"/>
+      <c r="G4" s="364"/>
+      <c r="H4" s="365"/>
+      <c r="I4" s="366"/>
+      <c r="J4" s="367"/>
+      <c r="K4" s="366"/>
+      <c r="L4" s="367"/>
+      <c r="M4" s="366"/>
+      <c r="N4" s="368"/>
     </row>
     <row r="5" spans="1:14" s="167" customFormat="1" ht="46.5" customHeight="1">
       <c r="A5" s="166">
         <v>1</v>
       </c>
-      <c r="B5" s="364" t="s">
+      <c r="B5" s="334" t="s">
         <v>154</v>
       </c>
-      <c r="C5" s="365"/>
-      <c r="D5" s="365"/>
-      <c r="E5" s="365"/>
-      <c r="F5" s="365"/>
-      <c r="G5" s="365"/>
-      <c r="H5" s="365"/>
-      <c r="I5" s="365"/>
-      <c r="J5" s="365"/>
-      <c r="K5" s="365"/>
-      <c r="L5" s="365"/>
-      <c r="M5" s="365"/>
-      <c r="N5" s="366"/>
+      <c r="C5" s="335"/>
+      <c r="D5" s="335"/>
+      <c r="E5" s="335"/>
+      <c r="F5" s="335"/>
+      <c r="G5" s="335"/>
+      <c r="H5" s="335"/>
+      <c r="I5" s="335"/>
+      <c r="J5" s="335"/>
+      <c r="K5" s="335"/>
+      <c r="L5" s="335"/>
+      <c r="M5" s="335"/>
+      <c r="N5" s="336"/>
     </row>
     <row r="6" spans="1:14" s="167" customFormat="1" ht="39" customHeight="1">
       <c r="A6" s="168">
         <v>2</v>
       </c>
-      <c r="B6" s="367" t="s">
+      <c r="B6" s="337" t="s">
         <v>155</v>
       </c>
-      <c r="C6" s="368"/>
-      <c r="D6" s="368"/>
-      <c r="E6" s="368"/>
-      <c r="F6" s="368"/>
-      <c r="G6" s="368"/>
-      <c r="H6" s="368"/>
-      <c r="I6" s="368"/>
-      <c r="J6" s="368"/>
-      <c r="K6" s="368"/>
-      <c r="L6" s="368"/>
-      <c r="M6" s="368"/>
-      <c r="N6" s="369"/>
+      <c r="C6" s="338"/>
+      <c r="D6" s="338"/>
+      <c r="E6" s="338"/>
+      <c r="F6" s="338"/>
+      <c r="G6" s="338"/>
+      <c r="H6" s="338"/>
+      <c r="I6" s="338"/>
+      <c r="J6" s="338"/>
+      <c r="K6" s="338"/>
+      <c r="L6" s="338"/>
+      <c r="M6" s="338"/>
+      <c r="N6" s="339"/>
     </row>
     <row r="7" spans="1:14" s="167" customFormat="1" ht="21" customHeight="1">
       <c r="A7" s="169" t="s">
         <v>156</v>
       </c>
-      <c r="B7" s="370" t="s">
+      <c r="B7" s="340" t="s">
         <v>157</v>
       </c>
-      <c r="C7" s="371"/>
-      <c r="D7" s="371"/>
-      <c r="E7" s="371"/>
-      <c r="F7" s="371"/>
-      <c r="G7" s="371"/>
-      <c r="H7" s="371"/>
-      <c r="I7" s="371"/>
-      <c r="J7" s="371"/>
-      <c r="K7" s="371"/>
-      <c r="L7" s="371"/>
-      <c r="M7" s="371"/>
-      <c r="N7" s="372"/>
+      <c r="C7" s="341"/>
+      <c r="D7" s="341"/>
+      <c r="E7" s="341"/>
+      <c r="F7" s="341"/>
+      <c r="G7" s="341"/>
+      <c r="H7" s="341"/>
+      <c r="I7" s="341"/>
+      <c r="J7" s="341"/>
+      <c r="K7" s="341"/>
+      <c r="L7" s="341"/>
+      <c r="M7" s="341"/>
+      <c r="N7" s="342"/>
     </row>
     <row r="8" spans="1:14" s="174" customFormat="1" ht="20.100000000000001" customHeight="1">
       <c r="A8" s="170"/>
@@ -38992,7 +38995,7 @@
       <c r="N42" s="178"/>
     </row>
     <row r="43" spans="1:14" s="202" customFormat="1" ht="18.75" customHeight="1">
-      <c r="A43" s="373" t="s">
+      <c r="A43" s="343" t="s">
         <v>162</v>
       </c>
       <c r="B43" s="195" t="s">
@@ -39000,81 +39003,95 @@
       </c>
       <c r="C43" s="196"/>
       <c r="D43" s="197"/>
-      <c r="E43" s="376"/>
-      <c r="F43" s="377"/>
-      <c r="G43" s="377"/>
-      <c r="H43" s="377"/>
-      <c r="I43" s="377"/>
-      <c r="J43" s="377"/>
+      <c r="E43" s="346"/>
+      <c r="F43" s="347"/>
+      <c r="G43" s="347"/>
+      <c r="H43" s="347"/>
+      <c r="I43" s="347"/>
+      <c r="J43" s="347"/>
       <c r="K43" s="200"/>
       <c r="L43" s="199"/>
       <c r="M43" s="198"/>
       <c r="N43" s="201"/>
     </row>
     <row r="44" spans="1:14" s="202" customFormat="1" ht="18.75" customHeight="1">
-      <c r="A44" s="374"/>
+      <c r="A44" s="344"/>
       <c r="B44" s="203" t="s">
         <v>163</v>
       </c>
       <c r="C44" s="204"/>
       <c r="D44" s="205"/>
-      <c r="E44" s="378"/>
-      <c r="F44" s="379"/>
-      <c r="G44" s="379"/>
-      <c r="H44" s="379"/>
-      <c r="I44" s="379"/>
-      <c r="J44" s="379"/>
+      <c r="E44" s="348"/>
+      <c r="F44" s="349"/>
+      <c r="G44" s="349"/>
+      <c r="H44" s="349"/>
+      <c r="I44" s="349"/>
+      <c r="J44" s="349"/>
       <c r="K44" s="206"/>
       <c r="L44" s="207"/>
       <c r="M44" s="208"/>
       <c r="N44" s="209"/>
     </row>
     <row r="45" spans="1:14" s="202" customFormat="1" ht="18.75" customHeight="1">
-      <c r="A45" s="374"/>
+      <c r="A45" s="344"/>
       <c r="B45" s="210" t="s">
         <v>164</v>
       </c>
       <c r="C45" s="204"/>
       <c r="D45" s="205"/>
-      <c r="E45" s="380"/>
-      <c r="F45" s="381"/>
-      <c r="G45" s="381"/>
-      <c r="H45" s="381"/>
-      <c r="I45" s="381"/>
-      <c r="J45" s="381"/>
+      <c r="E45" s="350"/>
+      <c r="F45" s="351"/>
+      <c r="G45" s="351"/>
+      <c r="H45" s="351"/>
+      <c r="I45" s="351"/>
+      <c r="J45" s="351"/>
       <c r="K45" s="211"/>
       <c r="L45" s="207"/>
       <c r="M45" s="212"/>
       <c r="N45" s="213"/>
     </row>
     <row r="46" spans="1:14" s="202" customFormat="1" ht="25.5" customHeight="1" thickBot="1">
-      <c r="A46" s="375"/>
+      <c r="A46" s="345"/>
       <c r="B46" s="214" t="s">
         <v>165</v>
       </c>
-      <c r="C46" s="382" t="s">
+      <c r="C46" s="352" t="s">
         <v>166</v>
       </c>
-      <c r="D46" s="383"/>
-      <c r="E46" s="384" t="s">
+      <c r="D46" s="353"/>
+      <c r="E46" s="354" t="s">
         <v>167</v>
       </c>
-      <c r="F46" s="385"/>
-      <c r="G46" s="385"/>
-      <c r="H46" s="385"/>
-      <c r="I46" s="385"/>
-      <c r="J46" s="386"/>
-      <c r="K46" s="362" t="s">
+      <c r="F46" s="355"/>
+      <c r="G46" s="355"/>
+      <c r="H46" s="355"/>
+      <c r="I46" s="355"/>
+      <c r="J46" s="356"/>
+      <c r="K46" s="332" t="s">
         <v>168</v>
       </c>
-      <c r="L46" s="386"/>
-      <c r="M46" s="362" t="s">
+      <c r="L46" s="356"/>
+      <c r="M46" s="332" t="s">
         <v>169</v>
       </c>
-      <c r="N46" s="363"/>
+      <c r="N46" s="333"/>
     </row>
   </sheetData>
   <mergeCells count="25">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="L1:N1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="L2:N2"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="I3:J3"/>
+    <mergeCell ref="K3:L3"/>
+    <mergeCell ref="M3:N3"/>
+    <mergeCell ref="B4:H4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="M4:N4"/>
     <mergeCell ref="M46:N46"/>
     <mergeCell ref="B5:N5"/>
     <mergeCell ref="B6:N6"/>
@@ -39086,20 +39103,6 @@
     <mergeCell ref="C46:D46"/>
     <mergeCell ref="E46:J46"/>
     <mergeCell ref="K46:L46"/>
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="I3:J3"/>
-    <mergeCell ref="K3:L3"/>
-    <mergeCell ref="M3:N3"/>
-    <mergeCell ref="B4:H4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="M4:N4"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="I1:K1"/>
-    <mergeCell ref="L1:N1"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="L2:N2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -40719,6 +40722,11 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="A52:B52"/>
+    <mergeCell ref="C52:D52"/>
+    <mergeCell ref="E52:F52"/>
+    <mergeCell ref="G52:I52"/>
+    <mergeCell ref="G57:I57"/>
     <mergeCell ref="A49:B49"/>
     <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:L3"/>
@@ -40732,11 +40740,6 @@
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="G11:H11"/>
     <mergeCell ref="I4:J4"/>
-    <mergeCell ref="A52:B52"/>
-    <mergeCell ref="C52:D52"/>
-    <mergeCell ref="E52:F52"/>
-    <mergeCell ref="G52:I52"/>
-    <mergeCell ref="G57:I57"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="68" orientation="portrait" r:id="rId1"/>
@@ -42684,6 +42687,16 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="K9:L9"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="E10:E11"/>
+    <mergeCell ref="G10:H10"/>
+    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="K5:L5"/>
+    <mergeCell ref="I6:J6"/>
     <mergeCell ref="G65:I65"/>
     <mergeCell ref="A58:B58"/>
     <mergeCell ref="C11:D11"/>
@@ -42692,16 +42705,6 @@
     <mergeCell ref="C60:D60"/>
     <mergeCell ref="E60:F60"/>
     <mergeCell ref="G60:I60"/>
-    <mergeCell ref="A3:L3"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="K5:L5"/>
-    <mergeCell ref="I6:J6"/>
-    <mergeCell ref="J9:J10"/>
-    <mergeCell ref="K9:L9"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="E10:E11"/>
-    <mergeCell ref="G10:H10"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="68" orientation="portrait" r:id="rId1"/>

</xml_diff>